<commit_message>
finishing parameters before run
</commit_message>
<xml_diff>
--- a/code/resultados/NWJSSP_OADG_BRKGA.xlsx
+++ b/code/resultados/NWJSSP_OADG_BRKGA.xlsx
@@ -1032,24 +1032,6 @@
       <c r="B1" t="n">
         <v>93.10914921760559</v>
       </c>
-      <c r="C1" t="inlineStr"/>
-      <c r="D1" t="inlineStr"/>
-      <c r="E1" t="inlineStr"/>
-      <c r="F1" t="inlineStr"/>
-      <c r="G1" t="inlineStr"/>
-      <c r="H1" t="inlineStr"/>
-      <c r="I1" t="inlineStr"/>
-      <c r="J1" t="inlineStr"/>
-      <c r="K1" t="inlineStr"/>
-      <c r="L1" t="inlineStr"/>
-      <c r="M1" t="inlineStr"/>
-      <c r="N1" t="inlineStr"/>
-      <c r="O1" t="inlineStr"/>
-      <c r="P1" t="inlineStr"/>
-      <c r="Q1" t="inlineStr"/>
-      <c r="R1" t="inlineStr"/>
-      <c r="S1" t="inlineStr"/>
-      <c r="T1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -1129,42 +1111,50 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>94122</v>
+        <v>95507</v>
       </c>
       <c r="B1" t="n">
-        <v>-1779213478791</v>
-      </c>
+        <v>50.44834065437317</v>
+      </c>
+      <c r="C1" t="inlineStr"/>
+      <c r="D1" t="inlineStr"/>
+      <c r="E1" t="inlineStr"/>
+      <c r="F1" t="inlineStr"/>
+      <c r="G1" t="inlineStr"/>
+      <c r="H1" t="inlineStr"/>
+      <c r="I1" t="inlineStr"/>
+      <c r="J1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="n">
+        <v>712</v>
+      </c>
+      <c r="B2" t="n">
+        <v>2031</v>
+      </c>
+      <c r="C2" t="n">
+        <v>848</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3026</v>
+      </c>
+      <c r="E2" t="n">
+        <v>6725</v>
+      </c>
+      <c r="F2" t="n">
+        <v>11551</v>
+      </c>
+      <c r="G2" t="n">
+        <v>4661</v>
+      </c>
+      <c r="H2" t="n">
+        <v>5538</v>
+      </c>
+      <c r="I2" t="n">
+        <v>7660</v>
+      </c>
+      <c r="J2" t="n">
         <v>0</v>
-      </c>
-      <c r="B2" t="n">
-        <v>118</v>
-      </c>
-      <c r="C2" t="n">
-        <v>4829</v>
-      </c>
-      <c r="D2" t="n">
-        <v>7278</v>
-      </c>
-      <c r="E2" t="n">
-        <v>5204</v>
-      </c>
-      <c r="F2" t="n">
-        <v>8183</v>
-      </c>
-      <c r="G2" t="n">
-        <v>3140</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>8786</v>
-      </c>
-      <c r="J2" t="n">
-        <v>3829</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new results, correct time e;apsed
</commit_message>
<xml_diff>
--- a/code/resultados/NWJSSP_OADG_BRKGA.xlsx
+++ b/code/resultados/NWJSSP_OADG_BRKGA.xlsx
@@ -430,7 +430,7 @@
         <v>308</v>
       </c>
       <c r="B1" t="n">
-        <v>3.230809926986694</v>
+        <v>3226</v>
       </c>
     </row>
     <row r="2">
@@ -469,312 +469,312 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>6439557</v>
+        <v>6639011</v>
       </c>
       <c r="B1" t="n">
-        <v>-1779213514141</v>
+        <v>3632.388556718826</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>14049</v>
+        <v>32611</v>
       </c>
       <c r="B2" t="n">
-        <v>102750</v>
+        <v>53915</v>
       </c>
       <c r="C2" t="n">
-        <v>91747</v>
+        <v>5669</v>
       </c>
       <c r="D2" t="n">
+        <v>49307</v>
+      </c>
+      <c r="E2" t="n">
+        <v>55449</v>
+      </c>
+      <c r="F2" t="n">
         <v>0</v>
       </c>
-      <c r="E2" t="n">
-        <v>57134</v>
-      </c>
-      <c r="F2" t="n">
-        <v>65613</v>
-      </c>
       <c r="G2" t="n">
-        <v>82975</v>
+        <v>33367</v>
       </c>
       <c r="H2" t="n">
-        <v>37862</v>
+        <v>112581</v>
       </c>
       <c r="I2" t="n">
-        <v>109799</v>
+        <v>45437</v>
       </c>
       <c r="J2" t="n">
-        <v>27405</v>
+        <v>15510</v>
       </c>
       <c r="K2" t="n">
-        <v>16325</v>
+        <v>92006</v>
       </c>
       <c r="L2" t="n">
-        <v>96232</v>
+        <v>117853</v>
       </c>
       <c r="M2" t="n">
-        <v>71381</v>
+        <v>111993</v>
       </c>
       <c r="N2" t="n">
-        <v>8660</v>
+        <v>72481</v>
       </c>
       <c r="O2" t="n">
-        <v>71575</v>
+        <v>115540</v>
       </c>
       <c r="P2" t="n">
-        <v>98908</v>
+        <v>2878</v>
       </c>
       <c r="Q2" t="n">
-        <v>5063</v>
+        <v>87446</v>
       </c>
       <c r="R2" t="n">
-        <v>118361</v>
+        <v>19536</v>
       </c>
       <c r="S2" t="n">
-        <v>119010</v>
+        <v>107277</v>
       </c>
       <c r="T2" t="n">
-        <v>13662</v>
+        <v>18679</v>
       </c>
       <c r="U2" t="n">
-        <v>60981</v>
+        <v>14144</v>
       </c>
       <c r="V2" t="n">
-        <v>0</v>
+        <v>43787</v>
       </c>
       <c r="W2" t="n">
-        <v>64421</v>
+        <v>135019</v>
       </c>
       <c r="X2" t="n">
-        <v>113158</v>
+        <v>57606</v>
       </c>
       <c r="Y2" t="n">
-        <v>76982</v>
+        <v>22053</v>
       </c>
       <c r="Z2" t="n">
-        <v>77648</v>
+        <v>116495</v>
       </c>
       <c r="AA2" t="n">
-        <v>80970</v>
+        <v>7319</v>
       </c>
       <c r="AB2" t="n">
-        <v>60876</v>
+        <v>58691</v>
       </c>
       <c r="AC2" t="n">
-        <v>56507</v>
+        <v>76986</v>
       </c>
       <c r="AD2" t="n">
-        <v>18844</v>
+        <v>17283</v>
       </c>
       <c r="AE2" t="n">
-        <v>122387</v>
+        <v>22218</v>
       </c>
       <c r="AF2" t="n">
-        <v>119813</v>
+        <v>120628</v>
       </c>
       <c r="AG2" t="n">
-        <v>45912</v>
+        <v>9119</v>
       </c>
       <c r="AH2" t="n">
-        <v>68427</v>
+        <v>128915</v>
       </c>
       <c r="AI2" t="n">
-        <v>27413</v>
+        <v>67330</v>
       </c>
       <c r="AJ2" t="n">
-        <v>60610</v>
+        <v>81968</v>
       </c>
       <c r="AK2" t="n">
-        <v>10812</v>
+        <v>61729</v>
       </c>
       <c r="AL2" t="n">
-        <v>67079</v>
+        <v>13238</v>
       </c>
       <c r="AM2" t="n">
-        <v>50522</v>
+        <v>63266</v>
       </c>
       <c r="AN2" t="n">
-        <v>88930</v>
+        <v>94956</v>
       </c>
       <c r="AO2" t="n">
-        <v>105181</v>
+        <v>42835</v>
       </c>
       <c r="AP2" t="n">
-        <v>86054</v>
+        <v>12313</v>
       </c>
       <c r="AQ2" t="n">
-        <v>113080</v>
+        <v>10800</v>
       </c>
       <c r="AR2" t="n">
-        <v>87412</v>
+        <v>73392</v>
       </c>
       <c r="AS2" t="n">
-        <v>56275</v>
+        <v>76729</v>
       </c>
       <c r="AT2" t="n">
-        <v>98475</v>
+        <v>97450</v>
       </c>
       <c r="AU2" t="n">
-        <v>33450</v>
+        <v>30628</v>
       </c>
       <c r="AV2" t="n">
-        <v>53683</v>
+        <v>544</v>
       </c>
       <c r="AW2" t="n">
-        <v>8481</v>
+        <v>86749</v>
       </c>
       <c r="AX2" t="n">
-        <v>74218</v>
+        <v>33825</v>
       </c>
       <c r="AY2" t="n">
-        <v>23075</v>
+        <v>129674</v>
       </c>
       <c r="AZ2" t="n">
-        <v>93127</v>
+        <v>37777</v>
       </c>
       <c r="BA2" t="n">
-        <v>104458</v>
+        <v>126410</v>
       </c>
       <c r="BB2" t="n">
-        <v>56996</v>
+        <v>40403</v>
       </c>
       <c r="BC2" t="n">
-        <v>25752</v>
+        <v>132572</v>
       </c>
       <c r="BD2" t="n">
-        <v>47339</v>
+        <v>94107</v>
       </c>
       <c r="BE2" t="n">
-        <v>1713</v>
+        <v>65183</v>
       </c>
       <c r="BF2" t="n">
-        <v>22820</v>
+        <v>88624</v>
       </c>
       <c r="BG2" t="n">
-        <v>19455</v>
+        <v>48090</v>
       </c>
       <c r="BH2" t="n">
-        <v>21232</v>
+        <v>104393</v>
       </c>
       <c r="BI2" t="n">
-        <v>17490</v>
+        <v>107742</v>
       </c>
       <c r="BJ2" t="n">
-        <v>54040</v>
+        <v>58202</v>
       </c>
       <c r="BK2" t="n">
-        <v>21335</v>
+        <v>7094</v>
       </c>
       <c r="BL2" t="n">
-        <v>43010</v>
+        <v>102183</v>
       </c>
       <c r="BM2" t="n">
-        <v>13633</v>
+        <v>4214</v>
       </c>
       <c r="BN2" t="n">
-        <v>67831</v>
+        <v>89350</v>
       </c>
       <c r="BO2" t="n">
-        <v>37753</v>
+        <v>100760</v>
       </c>
       <c r="BP2" t="n">
-        <v>30907</v>
+        <v>28433</v>
       </c>
       <c r="BQ2" t="n">
-        <v>108934</v>
+        <v>51919</v>
       </c>
       <c r="BR2" t="n">
-        <v>29669</v>
+        <v>131655</v>
       </c>
       <c r="BS2" t="n">
-        <v>50847</v>
+        <v>76045</v>
       </c>
       <c r="BT2" t="n">
-        <v>76329</v>
+        <v>82175</v>
       </c>
       <c r="BU2" t="n">
-        <v>73404</v>
+        <v>9204</v>
       </c>
       <c r="BV2" t="n">
-        <v>84832</v>
+        <v>70245</v>
       </c>
       <c r="BW2" t="n">
-        <v>8977</v>
+        <v>81082</v>
       </c>
       <c r="BX2" t="n">
-        <v>34007</v>
+        <v>40833</v>
       </c>
       <c r="BY2" t="n">
-        <v>36281</v>
+        <v>108118</v>
       </c>
       <c r="BZ2" t="n">
-        <v>43203</v>
+        <v>84993</v>
       </c>
       <c r="CA2" t="n">
-        <v>16420</v>
+        <v>39360</v>
       </c>
       <c r="CB2" t="n">
-        <v>118214</v>
+        <v>31666</v>
       </c>
       <c r="CC2" t="n">
-        <v>80011</v>
+        <v>489</v>
       </c>
       <c r="CD2" t="n">
-        <v>100851</v>
+        <v>51305</v>
       </c>
       <c r="CE2" t="n">
-        <v>4459</v>
+        <v>62471</v>
       </c>
       <c r="CF2" t="n">
-        <v>49356</v>
+        <v>26157</v>
       </c>
       <c r="CG2" t="n">
-        <v>79185</v>
+        <v>79396</v>
       </c>
       <c r="CH2" t="n">
-        <v>36384</v>
+        <v>37172</v>
       </c>
       <c r="CI2" t="n">
-        <v>93202</v>
+        <v>47223</v>
       </c>
       <c r="CJ2" t="n">
-        <v>39851</v>
+        <v>68774</v>
       </c>
       <c r="CK2" t="n">
-        <v>123228</v>
+        <v>45780</v>
       </c>
       <c r="CL2" t="n">
-        <v>30776</v>
+        <v>27720</v>
       </c>
       <c r="CM2" t="n">
-        <v>114883</v>
+        <v>122602</v>
       </c>
       <c r="CN2" t="n">
-        <v>127092</v>
+        <v>1657</v>
       </c>
       <c r="CO2" t="n">
-        <v>115679</v>
+        <v>115623</v>
       </c>
       <c r="CP2" t="n">
-        <v>41246</v>
+        <v>56994</v>
       </c>
       <c r="CQ2" t="n">
-        <v>6191</v>
+        <v>43220</v>
       </c>
       <c r="CR2" t="n">
-        <v>32499</v>
+        <v>24253</v>
       </c>
       <c r="CS2" t="n">
-        <v>103873</v>
+        <v>77501</v>
       </c>
       <c r="CT2" t="n">
-        <v>89719</v>
+        <v>125915</v>
       </c>
       <c r="CU2" t="n">
-        <v>44724</v>
+        <v>19757</v>
       </c>
       <c r="CV2" t="n">
-        <v>41327</v>
+        <v>100120</v>
       </c>
     </row>
   </sheetData>
@@ -796,7 +796,7 @@
         <v>321</v>
       </c>
       <c r="B1" t="n">
-        <v>2.338897943496704</v>
+        <v>2294</v>
       </c>
     </row>
     <row r="2">
@@ -835,24 +835,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>9814</v>
+        <v>9883</v>
       </c>
       <c r="B1" t="n">
-        <v>20.13490557670593</v>
+        <v>25945</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>486</v>
+        <v>834</v>
       </c>
       <c r="B2" t="n">
         <v>197</v>
       </c>
       <c r="C2" t="n">
-        <v>925</v>
+        <v>1097</v>
       </c>
       <c r="D2" t="n">
-        <v>725</v>
+        <v>941</v>
       </c>
       <c r="E2" t="n">
         <v>65</v>
@@ -864,10 +864,10 @@
         <v>209</v>
       </c>
       <c r="H2" t="n">
-        <v>562</v>
+        <v>602</v>
       </c>
       <c r="I2" t="n">
-        <v>1170</v>
+        <v>463</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -892,7 +892,7 @@
         <v>10203</v>
       </c>
       <c r="B1" t="n">
-        <v>40.17168784141541</v>
+        <v>26085</v>
       </c>
     </row>
     <row r="2">
@@ -943,72 +943,72 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>16955</v>
+        <v>17223</v>
       </c>
       <c r="B1" t="n">
-        <v>116.7028329372406</v>
+        <v>117172</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>167</v>
+        <v>7</v>
       </c>
       <c r="B2" t="n">
-        <v>874</v>
+        <v>152</v>
       </c>
       <c r="C2" t="n">
-        <v>1092</v>
+        <v>918</v>
       </c>
       <c r="D2" t="n">
-        <v>437</v>
+        <v>618</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>908</v>
+        <v>186</v>
       </c>
       <c r="G2" t="n">
         <v>45</v>
       </c>
       <c r="H2" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I2" t="n">
-        <v>985</v>
+        <v>1347</v>
       </c>
       <c r="J2" t="n">
-        <v>1262</v>
+        <v>791</v>
       </c>
       <c r="K2" t="n">
-        <v>241</v>
+        <v>345</v>
       </c>
       <c r="L2" t="n">
-        <v>254</v>
+        <v>385</v>
       </c>
       <c r="M2" t="n">
-        <v>403</v>
+        <v>590</v>
       </c>
       <c r="N2" t="n">
-        <v>1408</v>
+        <v>1332</v>
       </c>
       <c r="O2" t="n">
-        <v>627</v>
+        <v>1132</v>
       </c>
       <c r="P2" t="n">
-        <v>631</v>
+        <v>789</v>
       </c>
       <c r="Q2" t="n">
-        <v>366</v>
+        <v>510</v>
       </c>
       <c r="R2" t="n">
-        <v>1261</v>
+        <v>1203</v>
       </c>
       <c r="S2" t="n">
-        <v>743</v>
+        <v>1069</v>
       </c>
       <c r="T2" t="n">
-        <v>23</v>
+        <v>577</v>
       </c>
     </row>
   </sheetData>
@@ -1027,10 +1027,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>17911</v>
+        <v>18031</v>
       </c>
       <c r="B1" t="n">
-        <v>93.10914921760559</v>
+        <v>149632</v>
       </c>
     </row>
     <row r="2">
@@ -1041,10 +1041,10 @@
         <v>62</v>
       </c>
       <c r="C2" t="n">
-        <v>648</v>
+        <v>449</v>
       </c>
       <c r="D2" t="n">
-        <v>375</v>
+        <v>596</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -1056,40 +1056,40 @@
         <v>299</v>
       </c>
       <c r="H2" t="n">
-        <v>493</v>
+        <v>372</v>
       </c>
       <c r="I2" t="n">
-        <v>1541</v>
+        <v>1385</v>
       </c>
       <c r="J2" t="n">
-        <v>1136</v>
+        <v>911</v>
       </c>
       <c r="K2" t="n">
-        <v>570</v>
+        <v>786</v>
       </c>
       <c r="L2" t="n">
-        <v>638</v>
+        <v>439</v>
       </c>
       <c r="M2" t="n">
-        <v>1062</v>
+        <v>584</v>
       </c>
       <c r="N2" t="n">
-        <v>868</v>
+        <v>1376</v>
       </c>
       <c r="O2" t="n">
-        <v>827</v>
+        <v>1191</v>
       </c>
       <c r="P2" t="n">
-        <v>831</v>
+        <v>909</v>
       </c>
       <c r="Q2" t="n">
-        <v>406</v>
+        <v>829</v>
       </c>
       <c r="R2" t="n">
-        <v>1397</v>
+        <v>1241</v>
       </c>
       <c r="S2" t="n">
-        <v>1263</v>
+        <v>1107</v>
       </c>
       <c r="T2" t="n">
         <v>275</v>
@@ -1111,50 +1111,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>95507</v>
+        <v>94122</v>
       </c>
       <c r="B1" t="n">
-        <v>50.44834065437317</v>
-      </c>
-      <c r="C1" t="inlineStr"/>
-      <c r="D1" t="inlineStr"/>
-      <c r="E1" t="inlineStr"/>
-      <c r="F1" t="inlineStr"/>
-      <c r="G1" t="inlineStr"/>
-      <c r="H1" t="inlineStr"/>
-      <c r="I1" t="inlineStr"/>
-      <c r="J1" t="inlineStr"/>
+        <v>63552</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>712</v>
+        <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>2031</v>
+        <v>118</v>
       </c>
       <c r="C2" t="n">
-        <v>848</v>
+        <v>4829</v>
       </c>
       <c r="D2" t="n">
-        <v>3026</v>
+        <v>7278</v>
       </c>
       <c r="E2" t="n">
-        <v>6725</v>
+        <v>5204</v>
       </c>
       <c r="F2" t="n">
-        <v>11551</v>
+        <v>8183</v>
       </c>
       <c r="G2" t="n">
-        <v>4661</v>
+        <v>3140</v>
       </c>
       <c r="H2" t="n">
-        <v>5538</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>7660</v>
+        <v>8786</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>3829</v>
       </c>
     </row>
   </sheetData>
@@ -1176,8 +1168,16 @@
         <v>94122</v>
       </c>
       <c r="B1" t="n">
-        <v>-1779213491583</v>
-      </c>
+        <v>53959</v>
+      </c>
+      <c r="C1" t="inlineStr"/>
+      <c r="D1" t="inlineStr"/>
+      <c r="E1" t="inlineStr"/>
+      <c r="F1" t="inlineStr"/>
+      <c r="G1" t="inlineStr"/>
+      <c r="H1" t="inlineStr"/>
+      <c r="I1" t="inlineStr"/>
+      <c r="J1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -1227,312 +1227,312 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>6490716</v>
+        <v>6581176</v>
       </c>
       <c r="B1" t="n">
-        <v>-1779209886055</v>
+        <v>3644.367998361588</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>63772</v>
+        <v>4719</v>
       </c>
       <c r="B2" t="n">
-        <v>115347</v>
+        <v>73814</v>
       </c>
       <c r="C2" t="n">
-        <v>59616</v>
+        <v>69927</v>
       </c>
       <c r="D2" t="n">
-        <v>7554</v>
+        <v>66322</v>
       </c>
       <c r="E2" t="n">
-        <v>119282</v>
+        <v>114091</v>
       </c>
       <c r="F2" t="n">
-        <v>65786</v>
+        <v>59678</v>
       </c>
       <c r="G2" t="n">
-        <v>4387</v>
+        <v>51785</v>
       </c>
       <c r="H2" t="n">
-        <v>13967</v>
+        <v>44305</v>
       </c>
       <c r="I2" t="n">
-        <v>27830</v>
+        <v>18681</v>
       </c>
       <c r="J2" t="n">
-        <v>17094</v>
+        <v>55187</v>
       </c>
       <c r="K2" t="n">
-        <v>84810</v>
+        <v>30343</v>
       </c>
       <c r="L2" t="n">
-        <v>25231</v>
+        <v>50913</v>
       </c>
       <c r="M2" t="n">
-        <v>108094</v>
+        <v>81871</v>
       </c>
       <c r="N2" t="n">
-        <v>96622</v>
+        <v>7494</v>
       </c>
       <c r="O2" t="n">
-        <v>119116</v>
+        <v>118775</v>
       </c>
       <c r="P2" t="n">
-        <v>37379</v>
+        <v>56867</v>
       </c>
       <c r="Q2" t="n">
-        <v>121183</v>
+        <v>12912</v>
       </c>
       <c r="R2" t="n">
-        <v>10400</v>
+        <v>135455</v>
       </c>
       <c r="S2" t="n">
-        <v>59051</v>
+        <v>106890</v>
       </c>
       <c r="T2" t="n">
-        <v>44871</v>
+        <v>13165</v>
       </c>
       <c r="U2" t="n">
-        <v>29033</v>
+        <v>20995</v>
       </c>
       <c r="V2" t="n">
-        <v>121540</v>
+        <v>37075</v>
       </c>
       <c r="W2" t="n">
-        <v>33830</v>
+        <v>0</v>
       </c>
       <c r="X2" t="n">
-        <v>7781</v>
+        <v>38649</v>
       </c>
       <c r="Y2" t="n">
-        <v>94999</v>
+        <v>130725</v>
       </c>
       <c r="Z2" t="n">
-        <v>83247</v>
+        <v>93458</v>
       </c>
       <c r="AA2" t="n">
-        <v>89704</v>
+        <v>120462</v>
       </c>
       <c r="AB2" t="n">
-        <v>63516</v>
+        <v>103967</v>
       </c>
       <c r="AC2" t="n">
-        <v>21542</v>
+        <v>85119</v>
       </c>
       <c r="AD2" t="n">
-        <v>69825</v>
+        <v>39116</v>
       </c>
       <c r="AE2" t="n">
-        <v>103589</v>
+        <v>46037</v>
       </c>
       <c r="AF2" t="n">
-        <v>75500</v>
+        <v>2851</v>
       </c>
       <c r="AG2" t="n">
-        <v>74189</v>
+        <v>47527</v>
       </c>
       <c r="AH2" t="n">
+        <v>70050</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>125526</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>21112</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>6051</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>71066</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>34381</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>58432</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>76227</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>129114</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>94673</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>101355</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>41810</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>121895</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>119138</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>6326</v>
+      </c>
+      <c r="AW2" t="n">
+        <v>137413</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>124105</v>
+      </c>
+      <c r="AY2" t="n">
+        <v>63533</v>
+      </c>
+      <c r="AZ2" t="n">
+        <v>14183</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>97755</v>
+      </c>
+      <c r="BB2" t="n">
+        <v>26124</v>
+      </c>
+      <c r="BC2" t="n">
+        <v>78952</v>
+      </c>
+      <c r="BD2" t="n">
         <v>0</v>
       </c>
-      <c r="AI2" t="n">
-        <v>53787</v>
-      </c>
-      <c r="AJ2" t="n">
-        <v>4044</v>
-      </c>
-      <c r="AK2" t="n">
+      <c r="BE2" t="n">
+        <v>75859</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>85974</v>
+      </c>
+      <c r="BG2" t="n">
+        <v>64976</v>
+      </c>
+      <c r="BH2" t="n">
+        <v>111062</v>
+      </c>
+      <c r="BI2" t="n">
+        <v>16452</v>
+      </c>
+      <c r="BJ2" t="n">
+        <v>89336</v>
+      </c>
+      <c r="BK2" t="n">
+        <v>7833</v>
+      </c>
+      <c r="BL2" t="n">
+        <v>96732</v>
+      </c>
+      <c r="BM2" t="n">
+        <v>26724</v>
+      </c>
+      <c r="BN2" t="n">
+        <v>33513</v>
+      </c>
+      <c r="BO2" t="n">
+        <v>27885</v>
+      </c>
+      <c r="BP2" t="n">
+        <v>22735</v>
+      </c>
+      <c r="BQ2" t="n">
+        <v>50570</v>
+      </c>
+      <c r="BR2" t="n">
+        <v>11089</v>
+      </c>
+      <c r="BS2" t="n">
+        <v>30081</v>
+      </c>
+      <c r="BT2" t="n">
+        <v>80102</v>
+      </c>
+      <c r="BU2" t="n">
+        <v>61387</v>
+      </c>
+      <c r="BV2" t="n">
+        <v>3343</v>
+      </c>
+      <c r="BW2" t="n">
+        <v>16217</v>
+      </c>
+      <c r="BX2" t="n">
+        <v>20392</v>
+      </c>
+      <c r="BY2" t="n">
+        <v>127019</v>
+      </c>
+      <c r="BZ2" t="n">
+        <v>52499</v>
+      </c>
+      <c r="CA2" t="n">
+        <v>79835</v>
+      </c>
+      <c r="CB2" t="n">
+        <v>7952</v>
+      </c>
+      <c r="CC2" t="n">
+        <v>64771</v>
+      </c>
+      <c r="CD2" t="n">
+        <v>85345</v>
+      </c>
+      <c r="CE2" t="n">
+        <v>104381</v>
+      </c>
+      <c r="CF2" t="n">
+        <v>35120</v>
+      </c>
+      <c r="CG2" t="n">
+        <v>131397</v>
+      </c>
+      <c r="CH2" t="n">
+        <v>56376</v>
+      </c>
+      <c r="CI2" t="n">
+        <v>92030</v>
+      </c>
+      <c r="CJ2" t="n">
+        <v>14548</v>
+      </c>
+      <c r="CK2" t="n">
+        <v>114443</v>
+      </c>
+      <c r="CL2" t="n">
+        <v>24</v>
+      </c>
+      <c r="CM2" t="n">
+        <v>24558</v>
+      </c>
+      <c r="CN2" t="n">
         <v>55609</v>
       </c>
-      <c r="AL2" t="n">
-        <v>1888</v>
-      </c>
-      <c r="AM2" t="n">
-        <v>34846</v>
-      </c>
-      <c r="AN2" t="n">
-        <v>68514</v>
-      </c>
-      <c r="AO2" t="n">
-        <v>49902</v>
-      </c>
-      <c r="AP2" t="n">
-        <v>41430</v>
-      </c>
-      <c r="AQ2" t="n">
-        <v>79578</v>
-      </c>
-      <c r="AR2" t="n">
-        <v>44546</v>
-      </c>
-      <c r="AS2" t="n">
-        <v>75685</v>
-      </c>
-      <c r="AT2" t="n">
-        <v>124512</v>
-      </c>
-      <c r="AU2" t="n">
-        <v>85281</v>
-      </c>
-      <c r="AV2" t="n">
-        <v>30709</v>
-      </c>
-      <c r="AW2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX2" t="n">
-        <v>19713</v>
-      </c>
-      <c r="AY2" t="n">
-        <v>100233</v>
-      </c>
-      <c r="AZ2" t="n">
-        <v>47799</v>
-      </c>
-      <c r="BA2" t="n">
-        <v>88099</v>
-      </c>
-      <c r="BB2" t="n">
-        <v>35962</v>
-      </c>
-      <c r="BC2" t="n">
-        <v>105310</v>
-      </c>
-      <c r="BD2" t="n">
-        <v>51814</v>
-      </c>
-      <c r="BE2" t="n">
-        <v>729</v>
-      </c>
-      <c r="BF2" t="n">
-        <v>16608</v>
-      </c>
-      <c r="BG2" t="n">
-        <v>40656</v>
-      </c>
-      <c r="BH2" t="n">
-        <v>55954</v>
-      </c>
-      <c r="BI2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BJ2" t="n">
-        <v>114870</v>
-      </c>
-      <c r="BK2" t="n">
-        <v>26927</v>
-      </c>
-      <c r="BL2" t="n">
-        <v>73333</v>
-      </c>
-      <c r="BM2" t="n">
-        <v>112895</v>
-      </c>
-      <c r="BN2" t="n">
-        <v>70534</v>
-      </c>
-      <c r="BO2" t="n">
-        <v>18571</v>
-      </c>
-      <c r="BP2" t="n">
-        <v>67883</v>
-      </c>
-      <c r="BQ2" t="n">
-        <v>121525</v>
-      </c>
-      <c r="BR2" t="n">
-        <v>38465</v>
-      </c>
-      <c r="BS2" t="n">
-        <v>100703</v>
-      </c>
-      <c r="BT2" t="n">
-        <v>7343</v>
-      </c>
-      <c r="BU2" t="n">
-        <v>19260</v>
-      </c>
-      <c r="BV2" t="n">
-        <v>13568</v>
-      </c>
-      <c r="BW2" t="n">
-        <v>12665</v>
-      </c>
-      <c r="BX2" t="n">
-        <v>94239</v>
-      </c>
-      <c r="BY2" t="n">
-        <v>40567</v>
-      </c>
-      <c r="BZ2" t="n">
-        <v>103361</v>
-      </c>
-      <c r="CA2" t="n">
-        <v>22544</v>
-      </c>
-      <c r="CB2" t="n">
-        <v>91723</v>
-      </c>
-      <c r="CC2" t="n">
-        <v>62915</v>
-      </c>
-      <c r="CD2" t="n">
-        <v>126888</v>
-      </c>
-      <c r="CE2" t="n">
-        <v>78854</v>
-      </c>
-      <c r="CF2" t="n">
-        <v>97321</v>
-      </c>
-      <c r="CG2" t="n">
-        <v>43713</v>
-      </c>
-      <c r="CH2" t="n">
-        <v>106086</v>
-      </c>
-      <c r="CI2" t="n">
-        <v>69622</v>
-      </c>
-      <c r="CJ2" t="n">
-        <v>113110</v>
-      </c>
-      <c r="CK2" t="n">
-        <v>31291</v>
-      </c>
-      <c r="CL2" t="n">
-        <v>80408</v>
-      </c>
-      <c r="CM2" t="n">
-        <v>113920</v>
-      </c>
-      <c r="CN2" t="n">
-        <v>21570</v>
-      </c>
       <c r="CO2" t="n">
-        <v>108615</v>
+        <v>753</v>
       </c>
       <c r="CP2" t="n">
-        <v>60272</v>
+        <v>90966</v>
       </c>
       <c r="CQ2" t="n">
-        <v>29014</v>
+        <v>135125</v>
       </c>
       <c r="CR2" t="n">
-        <v>55656</v>
+        <v>31237</v>
       </c>
       <c r="CS2" t="n">
-        <v>48892</v>
+        <v>104569</v>
       </c>
       <c r="CT2" t="n">
-        <v>24377</v>
+        <v>41315</v>
       </c>
       <c r="CU2" t="n">
-        <v>92605</v>
+        <v>108704</v>
       </c>
       <c r="CV2" t="n">
-        <v>86890</v>
+        <v>27116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new epr.py added and results are nice
</commit_message>
<xml_diff>
--- a/code/resultados/NWJSSP_OADG_BRKGA.xlsx
+++ b/code/resultados/NWJSSP_OADG_BRKGA.xlsx
@@ -1170,14 +1170,6 @@
       <c r="B1" t="n">
         <v>53959</v>
       </c>
-      <c r="C1" t="inlineStr"/>
-      <c r="D1" t="inlineStr"/>
-      <c r="E1" t="inlineStr"/>
-      <c r="F1" t="inlineStr"/>
-      <c r="G1" t="inlineStr"/>
-      <c r="H1" t="inlineStr"/>
-      <c r="I1" t="inlineStr"/>
-      <c r="J1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -1227,312 +1219,410 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>6581176</v>
+        <v>6318254</v>
       </c>
       <c r="B1" t="n">
-        <v>3644.367998361588</v>
-      </c>
+        <v>3651579</v>
+      </c>
+      <c r="C1" t="inlineStr"/>
+      <c r="D1" t="inlineStr"/>
+      <c r="E1" t="inlineStr"/>
+      <c r="F1" t="inlineStr"/>
+      <c r="G1" t="inlineStr"/>
+      <c r="H1" t="inlineStr"/>
+      <c r="I1" t="inlineStr"/>
+      <c r="J1" t="inlineStr"/>
+      <c r="K1" t="inlineStr"/>
+      <c r="L1" t="inlineStr"/>
+      <c r="M1" t="inlineStr"/>
+      <c r="N1" t="inlineStr"/>
+      <c r="O1" t="inlineStr"/>
+      <c r="P1" t="inlineStr"/>
+      <c r="Q1" t="inlineStr"/>
+      <c r="R1" t="inlineStr"/>
+      <c r="S1" t="inlineStr"/>
+      <c r="T1" t="inlineStr"/>
+      <c r="U1" t="inlineStr"/>
+      <c r="V1" t="inlineStr"/>
+      <c r="W1" t="inlineStr"/>
+      <c r="X1" t="inlineStr"/>
+      <c r="Y1" t="inlineStr"/>
+      <c r="Z1" t="inlineStr"/>
+      <c r="AA1" t="inlineStr"/>
+      <c r="AB1" t="inlineStr"/>
+      <c r="AC1" t="inlineStr"/>
+      <c r="AD1" t="inlineStr"/>
+      <c r="AE1" t="inlineStr"/>
+      <c r="AF1" t="inlineStr"/>
+      <c r="AG1" t="inlineStr"/>
+      <c r="AH1" t="inlineStr"/>
+      <c r="AI1" t="inlineStr"/>
+      <c r="AJ1" t="inlineStr"/>
+      <c r="AK1" t="inlineStr"/>
+      <c r="AL1" t="inlineStr"/>
+      <c r="AM1" t="inlineStr"/>
+      <c r="AN1" t="inlineStr"/>
+      <c r="AO1" t="inlineStr"/>
+      <c r="AP1" t="inlineStr"/>
+      <c r="AQ1" t="inlineStr"/>
+      <c r="AR1" t="inlineStr"/>
+      <c r="AS1" t="inlineStr"/>
+      <c r="AT1" t="inlineStr"/>
+      <c r="AU1" t="inlineStr"/>
+      <c r="AV1" t="inlineStr"/>
+      <c r="AW1" t="inlineStr"/>
+      <c r="AX1" t="inlineStr"/>
+      <c r="AY1" t="inlineStr"/>
+      <c r="AZ1" t="inlineStr"/>
+      <c r="BA1" t="inlineStr"/>
+      <c r="BB1" t="inlineStr"/>
+      <c r="BC1" t="inlineStr"/>
+      <c r="BD1" t="inlineStr"/>
+      <c r="BE1" t="inlineStr"/>
+      <c r="BF1" t="inlineStr"/>
+      <c r="BG1" t="inlineStr"/>
+      <c r="BH1" t="inlineStr"/>
+      <c r="BI1" t="inlineStr"/>
+      <c r="BJ1" t="inlineStr"/>
+      <c r="BK1" t="inlineStr"/>
+      <c r="BL1" t="inlineStr"/>
+      <c r="BM1" t="inlineStr"/>
+      <c r="BN1" t="inlineStr"/>
+      <c r="BO1" t="inlineStr"/>
+      <c r="BP1" t="inlineStr"/>
+      <c r="BQ1" t="inlineStr"/>
+      <c r="BR1" t="inlineStr"/>
+      <c r="BS1" t="inlineStr"/>
+      <c r="BT1" t="inlineStr"/>
+      <c r="BU1" t="inlineStr"/>
+      <c r="BV1" t="inlineStr"/>
+      <c r="BW1" t="inlineStr"/>
+      <c r="BX1" t="inlineStr"/>
+      <c r="BY1" t="inlineStr"/>
+      <c r="BZ1" t="inlineStr"/>
+      <c r="CA1" t="inlineStr"/>
+      <c r="CB1" t="inlineStr"/>
+      <c r="CC1" t="inlineStr"/>
+      <c r="CD1" t="inlineStr"/>
+      <c r="CE1" t="inlineStr"/>
+      <c r="CF1" t="inlineStr"/>
+      <c r="CG1" t="inlineStr"/>
+      <c r="CH1" t="inlineStr"/>
+      <c r="CI1" t="inlineStr"/>
+      <c r="CJ1" t="inlineStr"/>
+      <c r="CK1" t="inlineStr"/>
+      <c r="CL1" t="inlineStr"/>
+      <c r="CM1" t="inlineStr"/>
+      <c r="CN1" t="inlineStr"/>
+      <c r="CO1" t="inlineStr"/>
+      <c r="CP1" t="inlineStr"/>
+      <c r="CQ1" t="inlineStr"/>
+      <c r="CR1" t="inlineStr"/>
+      <c r="CS1" t="inlineStr"/>
+      <c r="CT1" t="inlineStr"/>
+      <c r="CU1" t="inlineStr"/>
+      <c r="CV1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="n">
         <v>4719</v>
       </c>
       <c r="B2" t="n">
-        <v>73814</v>
+        <v>71268</v>
       </c>
       <c r="C2" t="n">
-        <v>69927</v>
+        <v>70778</v>
       </c>
       <c r="D2" t="n">
-        <v>66322</v>
+        <v>14873</v>
       </c>
       <c r="E2" t="n">
-        <v>114091</v>
+        <v>96495</v>
       </c>
       <c r="F2" t="n">
-        <v>59678</v>
+        <v>31497</v>
       </c>
       <c r="G2" t="n">
-        <v>51785</v>
+        <v>51628</v>
       </c>
       <c r="H2" t="n">
-        <v>44305</v>
+        <v>38548</v>
       </c>
       <c r="I2" t="n">
-        <v>18681</v>
+        <v>21114</v>
       </c>
       <c r="J2" t="n">
-        <v>55187</v>
+        <v>53817</v>
       </c>
       <c r="K2" t="n">
-        <v>30343</v>
+        <v>55444</v>
       </c>
       <c r="L2" t="n">
-        <v>50913</v>
+        <v>105682</v>
       </c>
       <c r="M2" t="n">
-        <v>81871</v>
+        <v>123412</v>
       </c>
       <c r="N2" t="n">
         <v>7494</v>
       </c>
       <c r="O2" t="n">
-        <v>118775</v>
+        <v>100004</v>
       </c>
       <c r="P2" t="n">
-        <v>56867</v>
+        <v>72824</v>
       </c>
       <c r="Q2" t="n">
-        <v>12912</v>
+        <v>55638</v>
       </c>
       <c r="R2" t="n">
-        <v>135455</v>
+        <v>107666</v>
       </c>
       <c r="S2" t="n">
-        <v>106890</v>
+        <v>90980</v>
       </c>
       <c r="T2" t="n">
-        <v>13165</v>
+        <v>11666</v>
       </c>
       <c r="U2" t="n">
-        <v>20995</v>
+        <v>25346</v>
       </c>
       <c r="V2" t="n">
-        <v>37075</v>
+        <v>34601</v>
       </c>
       <c r="W2" t="n">
         <v>0</v>
       </c>
       <c r="X2" t="n">
-        <v>38649</v>
+        <v>39945</v>
       </c>
       <c r="Y2" t="n">
-        <v>130725</v>
+        <v>37831</v>
       </c>
       <c r="Z2" t="n">
-        <v>93458</v>
+        <v>26444</v>
       </c>
       <c r="AA2" t="n">
-        <v>120462</v>
+        <v>102260</v>
       </c>
       <c r="AB2" t="n">
-        <v>103967</v>
+        <v>132224</v>
       </c>
       <c r="AC2" t="n">
-        <v>85119</v>
+        <v>15443</v>
       </c>
       <c r="AD2" t="n">
-        <v>39116</v>
+        <v>48606</v>
       </c>
       <c r="AE2" t="n">
-        <v>46037</v>
+        <v>43308</v>
       </c>
       <c r="AF2" t="n">
         <v>2851</v>
       </c>
       <c r="AG2" t="n">
-        <v>47527</v>
+        <v>50996</v>
       </c>
       <c r="AH2" t="n">
-        <v>70050</v>
+        <v>97860</v>
       </c>
       <c r="AI2" t="n">
-        <v>125526</v>
+        <v>110473</v>
       </c>
       <c r="AJ2" t="n">
-        <v>21112</v>
+        <v>19256</v>
       </c>
       <c r="AK2" t="n">
         <v>6051</v>
       </c>
       <c r="AL2" t="n">
-        <v>71066</v>
+        <v>67030</v>
       </c>
       <c r="AM2" t="n">
-        <v>34381</v>
+        <v>87029</v>
       </c>
       <c r="AN2" t="n">
-        <v>58432</v>
+        <v>56748</v>
       </c>
       <c r="AO2" t="n">
-        <v>76227</v>
+        <v>70321</v>
       </c>
       <c r="AP2" t="n">
-        <v>129114</v>
+        <v>120958</v>
       </c>
       <c r="AQ2" t="n">
-        <v>94673</v>
+        <v>83234</v>
       </c>
       <c r="AR2" t="n">
-        <v>101355</v>
+        <v>89916</v>
       </c>
       <c r="AS2" t="n">
-        <v>41810</v>
+        <v>14820</v>
       </c>
       <c r="AT2" t="n">
-        <v>121895</v>
+        <v>114996</v>
       </c>
       <c r="AU2" t="n">
-        <v>119138</v>
+        <v>100642</v>
       </c>
       <c r="AV2" t="n">
         <v>6326</v>
       </c>
       <c r="AW2" t="n">
-        <v>137413</v>
+        <v>132500</v>
       </c>
       <c r="AX2" t="n">
-        <v>124105</v>
+        <v>117206</v>
       </c>
       <c r="AY2" t="n">
-        <v>63533</v>
+        <v>61849</v>
       </c>
       <c r="AZ2" t="n">
-        <v>14183</v>
+        <v>26988</v>
       </c>
       <c r="BA2" t="n">
-        <v>97755</v>
+        <v>86316</v>
       </c>
       <c r="BB2" t="n">
-        <v>26124</v>
+        <v>12791</v>
       </c>
       <c r="BC2" t="n">
-        <v>78952</v>
+        <v>55484</v>
       </c>
       <c r="BD2" t="n">
         <v>0</v>
       </c>
       <c r="BE2" t="n">
-        <v>75859</v>
+        <v>20384</v>
       </c>
       <c r="BF2" t="n">
-        <v>85974</v>
+        <v>75893</v>
       </c>
       <c r="BG2" t="n">
-        <v>64976</v>
+        <v>62995</v>
       </c>
       <c r="BH2" t="n">
-        <v>111062</v>
+        <v>82833</v>
       </c>
       <c r="BI2" t="n">
-        <v>16452</v>
+        <v>95178</v>
       </c>
       <c r="BJ2" t="n">
-        <v>89336</v>
+        <v>80349</v>
       </c>
       <c r="BK2" t="n">
         <v>7833</v>
       </c>
       <c r="BL2" t="n">
-        <v>96732</v>
+        <v>85293</v>
       </c>
       <c r="BM2" t="n">
-        <v>26724</v>
+        <v>109009</v>
       </c>
       <c r="BN2" t="n">
-        <v>33513</v>
+        <v>31582</v>
       </c>
       <c r="BO2" t="n">
-        <v>27885</v>
+        <v>23786</v>
       </c>
       <c r="BP2" t="n">
-        <v>22735</v>
+        <v>21529</v>
       </c>
       <c r="BQ2" t="n">
-        <v>50570</v>
+        <v>43787</v>
       </c>
       <c r="BR2" t="n">
-        <v>11089</v>
+        <v>13646</v>
       </c>
       <c r="BS2" t="n">
-        <v>30081</v>
+        <v>28924</v>
       </c>
       <c r="BT2" t="n">
-        <v>80102</v>
+        <v>47370</v>
       </c>
       <c r="BU2" t="n">
-        <v>61387</v>
+        <v>59703</v>
       </c>
       <c r="BV2" t="n">
         <v>3343</v>
       </c>
       <c r="BW2" t="n">
-        <v>16217</v>
+        <v>45783</v>
       </c>
       <c r="BX2" t="n">
-        <v>20392</v>
+        <v>30113</v>
       </c>
       <c r="BY2" t="n">
-        <v>127019</v>
+        <v>120120</v>
       </c>
       <c r="BZ2" t="n">
-        <v>52499</v>
+        <v>104726</v>
       </c>
       <c r="CA2" t="n">
-        <v>79835</v>
+        <v>129735</v>
       </c>
       <c r="CB2" t="n">
         <v>7952</v>
       </c>
       <c r="CC2" t="n">
-        <v>64771</v>
+        <v>125476</v>
       </c>
       <c r="CD2" t="n">
-        <v>85345</v>
+        <v>17370</v>
       </c>
       <c r="CE2" t="n">
-        <v>104381</v>
+        <v>108434</v>
       </c>
       <c r="CF2" t="n">
-        <v>35120</v>
+        <v>74083</v>
       </c>
       <c r="CG2" t="n">
-        <v>131397</v>
+        <v>124195</v>
       </c>
       <c r="CH2" t="n">
-        <v>56376</v>
+        <v>37445</v>
       </c>
       <c r="CI2" t="n">
-        <v>92030</v>
+        <v>78746</v>
       </c>
       <c r="CJ2" t="n">
-        <v>14548</v>
+        <v>15417</v>
       </c>
       <c r="CK2" t="n">
-        <v>114443</v>
+        <v>66225</v>
       </c>
       <c r="CL2" t="n">
         <v>24</v>
       </c>
       <c r="CM2" t="n">
-        <v>24558</v>
+        <v>73832</v>
       </c>
       <c r="CN2" t="n">
-        <v>55609</v>
+        <v>78363</v>
       </c>
       <c r="CO2" t="n">
         <v>753</v>
       </c>
       <c r="CP2" t="n">
-        <v>90966</v>
+        <v>10982</v>
       </c>
       <c r="CQ2" t="n">
-        <v>135125</v>
+        <v>49300</v>
       </c>
       <c r="CR2" t="n">
-        <v>31237</v>
+        <v>31155</v>
       </c>
       <c r="CS2" t="n">
-        <v>104569</v>
+        <v>93283</v>
       </c>
       <c r="CT2" t="n">
-        <v>41315</v>
+        <v>35405</v>
       </c>
       <c r="CU2" t="n">
-        <v>108704</v>
+        <v>112838</v>
       </c>
       <c r="CV2" t="n">
-        <v>27116</v>
+        <v>64040</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new epr and new results
</commit_message>
<xml_diff>
--- a/code/resultados/NWJSSP_OADG_BRKGA.xlsx
+++ b/code/resultados/NWJSSP_OADG_BRKGA.xlsx
@@ -17,6 +17,8 @@
     <sheet name="tai_j10_m10_1r" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="tai_j100_m10_1" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="tai_j100_m10_1r" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="tai_j100_m100_1" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="tai_j100_m100_1r" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -474,6 +476,654 @@
       <c r="B1" t="n">
         <v>3614722</v>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>33729</v>
+      </c>
+      <c r="B2" t="n">
+        <v>53695</v>
+      </c>
+      <c r="C2" t="n">
+        <v>70605</v>
+      </c>
+      <c r="D2" t="n">
+        <v>48865</v>
+      </c>
+      <c r="E2" t="n">
+        <v>44191</v>
+      </c>
+      <c r="F2" t="n">
+        <v>54993</v>
+      </c>
+      <c r="G2" t="n">
+        <v>80596</v>
+      </c>
+      <c r="H2" t="n">
+        <v>20815</v>
+      </c>
+      <c r="I2" t="n">
+        <v>97301</v>
+      </c>
+      <c r="J2" t="n">
+        <v>44675</v>
+      </c>
+      <c r="K2" t="n">
+        <v>114261</v>
+      </c>
+      <c r="L2" t="n">
+        <v>5065</v>
+      </c>
+      <c r="M2" t="n">
+        <v>97492</v>
+      </c>
+      <c r="N2" t="n">
+        <v>82203</v>
+      </c>
+      <c r="O2" t="n">
+        <v>93985</v>
+      </c>
+      <c r="P2" t="n">
+        <v>49063</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>47242</v>
+      </c>
+      <c r="R2" t="n">
+        <v>10631</v>
+      </c>
+      <c r="S2" t="n">
+        <v>28389</v>
+      </c>
+      <c r="T2" t="n">
+        <v>65955</v>
+      </c>
+      <c r="U2" t="n">
+        <v>20619</v>
+      </c>
+      <c r="V2" t="n">
+        <v>124725</v>
+      </c>
+      <c r="W2" t="n">
+        <v>24543</v>
+      </c>
+      <c r="X2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>62541</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>10961</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>87159</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>865</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>53599</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>126</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>59744</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>126355</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>76232</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>66149</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>93134</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>74327</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>63316</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>119564</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>89070</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>100908</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>70978</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>28379</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>78993</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>84607</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>98471</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>103129</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>107829</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>93107</v>
+      </c>
+      <c r="AW2" t="n">
+        <v>66967</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>59474</v>
+      </c>
+      <c r="AY2" t="n">
+        <v>38913</v>
+      </c>
+      <c r="AZ2" t="n">
+        <v>5642</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>120143</v>
+      </c>
+      <c r="BB2" t="n">
+        <v>35039</v>
+      </c>
+      <c r="BC2" t="n">
+        <v>116512</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>25749</v>
+      </c>
+      <c r="BE2" t="n">
+        <v>28506</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>72483</v>
+      </c>
+      <c r="BG2" t="n">
+        <v>13784</v>
+      </c>
+      <c r="BH2" t="n">
+        <v>41752</v>
+      </c>
+      <c r="BI2" t="n">
+        <v>28947</v>
+      </c>
+      <c r="BJ2" t="n">
+        <v>16433</v>
+      </c>
+      <c r="BK2" t="n">
+        <v>16481</v>
+      </c>
+      <c r="BL2" t="n">
+        <v>49973</v>
+      </c>
+      <c r="BM2" t="n">
+        <v>107018</v>
+      </c>
+      <c r="BN2" t="n">
+        <v>35814</v>
+      </c>
+      <c r="BO2" t="n">
+        <v>20030</v>
+      </c>
+      <c r="BP2" t="n">
+        <v>38728</v>
+      </c>
+      <c r="BQ2" t="n">
+        <v>30624</v>
+      </c>
+      <c r="BR2" t="n">
+        <v>6052</v>
+      </c>
+      <c r="BS2" t="n">
+        <v>121882</v>
+      </c>
+      <c r="BT2" t="n">
+        <v>42103</v>
+      </c>
+      <c r="BU2" t="n">
+        <v>24950</v>
+      </c>
+      <c r="BV2" t="n">
+        <v>115799</v>
+      </c>
+      <c r="BW2" t="n">
+        <v>15994</v>
+      </c>
+      <c r="BX2" t="n">
+        <v>45938</v>
+      </c>
+      <c r="BY2" t="n">
+        <v>87813</v>
+      </c>
+      <c r="BZ2" t="n">
+        <v>6680</v>
+      </c>
+      <c r="CA2" t="n">
+        <v>459</v>
+      </c>
+      <c r="CB2" t="n">
+        <v>12877</v>
+      </c>
+      <c r="CC2" t="n">
+        <v>86093</v>
+      </c>
+      <c r="CD2" t="n">
+        <v>64985</v>
+      </c>
+      <c r="CE2" t="n">
+        <v>111461</v>
+      </c>
+      <c r="CF2" t="n">
+        <v>58149</v>
+      </c>
+      <c r="CG2" t="n">
+        <v>9455</v>
+      </c>
+      <c r="CH2" t="n">
+        <v>19337</v>
+      </c>
+      <c r="CI2" t="n">
+        <v>83255</v>
+      </c>
+      <c r="CJ2" t="n">
+        <v>113044</v>
+      </c>
+      <c r="CK2" t="n">
+        <v>39530</v>
+      </c>
+      <c r="CL2" t="n">
+        <v>2889</v>
+      </c>
+      <c r="CM2" t="n">
+        <v>77648</v>
+      </c>
+      <c r="CN2" t="n">
+        <v>57372</v>
+      </c>
+      <c r="CO2" t="n">
+        <v>105456</v>
+      </c>
+      <c r="CP2" t="n">
+        <v>81409</v>
+      </c>
+      <c r="CQ2" t="n">
+        <v>108994</v>
+      </c>
+      <c r="CR2" t="n">
+        <v>49638</v>
+      </c>
+      <c r="CS2" t="n">
+        <v>33110</v>
+      </c>
+      <c r="CT2" t="n">
+        <v>10341</v>
+      </c>
+      <c r="CU2" t="n">
+        <v>22740</v>
+      </c>
+      <c r="CV2" t="n">
+        <v>91812</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:CV2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="n">
+        <v>43470943</v>
+      </c>
+      <c r="B1" t="n">
+        <v>4577840</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>616769</v>
+      </c>
+      <c r="B2" t="n">
+        <v>701676</v>
+      </c>
+      <c r="C2" t="n">
+        <v>105574</v>
+      </c>
+      <c r="D2" t="n">
+        <v>63797</v>
+      </c>
+      <c r="E2" t="n">
+        <v>318151</v>
+      </c>
+      <c r="F2" t="n">
+        <v>181590</v>
+      </c>
+      <c r="G2" t="n">
+        <v>673373</v>
+      </c>
+      <c r="H2" t="n">
+        <v>450641</v>
+      </c>
+      <c r="I2" t="n">
+        <v>248670</v>
+      </c>
+      <c r="J2" t="n">
+        <v>742073</v>
+      </c>
+      <c r="K2" t="n">
+        <v>519730</v>
+      </c>
+      <c r="L2" t="n">
+        <v>502030</v>
+      </c>
+      <c r="M2" t="n">
+        <v>749100</v>
+      </c>
+      <c r="N2" t="n">
+        <v>465421</v>
+      </c>
+      <c r="O2" t="n">
+        <v>485204</v>
+      </c>
+      <c r="P2" t="n">
+        <v>38928</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>23327</v>
+      </c>
+      <c r="R2" t="n">
+        <v>326696</v>
+      </c>
+      <c r="S2" t="n">
+        <v>600466</v>
+      </c>
+      <c r="T2" t="n">
+        <v>729950</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V2" t="n">
+        <v>634600</v>
+      </c>
+      <c r="W2" t="n">
+        <v>615790</v>
+      </c>
+      <c r="X2" t="n">
+        <v>85681</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>922</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>784078</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>413607</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>147942</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>53386</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>761058</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>675764</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>379713</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>785522</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>519424</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>760036</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>740832</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>566812</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>28179</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>305152</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>646807</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>654480</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>557919</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>402954</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>219769</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>71471</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>559134</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>215606</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>226577</v>
+      </c>
+      <c r="AW2" t="n">
+        <v>10537</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>787550</v>
+      </c>
+      <c r="AY2" t="n">
+        <v>160932</v>
+      </c>
+      <c r="AZ2" t="n">
+        <v>25139</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>171556</v>
+      </c>
+      <c r="BB2" t="n">
+        <v>463072</v>
+      </c>
+      <c r="BC2" t="n">
+        <v>496202</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>534523</v>
+      </c>
+      <c r="BE2" t="n">
+        <v>365686</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>282981</v>
+      </c>
+      <c r="BG2" t="n">
+        <v>386227</v>
+      </c>
+      <c r="BH2" t="n">
+        <v>262079</v>
+      </c>
+      <c r="BI2" t="n">
+        <v>584793</v>
+      </c>
+      <c r="BJ2" t="n">
+        <v>562231</v>
+      </c>
+      <c r="BK2" t="n">
+        <v>80504</v>
+      </c>
+      <c r="BL2" t="n">
+        <v>204873</v>
+      </c>
+      <c r="BM2" t="n">
+        <v>336453</v>
+      </c>
+      <c r="BN2" t="n">
+        <v>237183</v>
+      </c>
+      <c r="BO2" t="n">
+        <v>131331</v>
+      </c>
+      <c r="BP2" t="n">
+        <v>493925</v>
+      </c>
+      <c r="BQ2" t="n">
+        <v>112644</v>
+      </c>
+      <c r="BR2" t="n">
+        <v>588187</v>
+      </c>
+      <c r="BS2" t="n">
+        <v>539337</v>
+      </c>
+      <c r="BT2" t="n">
+        <v>353666</v>
+      </c>
+      <c r="BU2" t="n">
+        <v>418829</v>
+      </c>
+      <c r="BV2" t="n">
+        <v>701741</v>
+      </c>
+      <c r="BW2" t="n">
+        <v>402149</v>
+      </c>
+      <c r="BX2" t="n">
+        <v>453534</v>
+      </c>
+      <c r="BY2" t="n">
+        <v>294413</v>
+      </c>
+      <c r="BZ2" t="n">
+        <v>103082</v>
+      </c>
+      <c r="CA2" t="n">
+        <v>387288</v>
+      </c>
+      <c r="CB2" t="n">
+        <v>819588</v>
+      </c>
+      <c r="CC2" t="n">
+        <v>350158</v>
+      </c>
+      <c r="CD2" t="n">
+        <v>127203</v>
+      </c>
+      <c r="CE2" t="n">
+        <v>420036</v>
+      </c>
+      <c r="CF2" t="n">
+        <v>279940</v>
+      </c>
+      <c r="CG2" t="n">
+        <v>159376</v>
+      </c>
+      <c r="CH2" t="n">
+        <v>3576</v>
+      </c>
+      <c r="CI2" t="n">
+        <v>102261</v>
+      </c>
+      <c r="CJ2" t="n">
+        <v>161264</v>
+      </c>
+      <c r="CK2" t="n">
+        <v>434412</v>
+      </c>
+      <c r="CL2" t="n">
+        <v>187678</v>
+      </c>
+      <c r="CM2" t="n">
+        <v>487016</v>
+      </c>
+      <c r="CN2" t="n">
+        <v>268026</v>
+      </c>
+      <c r="CO2" t="n">
+        <v>353998</v>
+      </c>
+      <c r="CP2" t="n">
+        <v>738027</v>
+      </c>
+      <c r="CQ2" t="n">
+        <v>308644</v>
+      </c>
+      <c r="CR2" t="n">
+        <v>133158</v>
+      </c>
+      <c r="CS2" t="n">
+        <v>199337</v>
+      </c>
+      <c r="CT2" t="n">
+        <v>708015</v>
+      </c>
+      <c r="CU2" t="n">
+        <v>695233</v>
+      </c>
+      <c r="CV2" t="n">
+        <v>246301</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:CV2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="n">
+        <v>44086748</v>
+      </c>
+      <c r="B1" t="n">
+        <v>4498508</v>
+      </c>
       <c r="C1" t="inlineStr"/>
       <c r="D1" t="inlineStr"/>
       <c r="E1" t="inlineStr"/>
@@ -575,304 +1225,304 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>33729</v>
+        <v>608588</v>
       </c>
       <c r="B2" t="n">
-        <v>53695</v>
+        <v>818806</v>
       </c>
       <c r="C2" t="n">
-        <v>70605</v>
+        <v>542197</v>
       </c>
       <c r="D2" t="n">
-        <v>48865</v>
+        <v>485751</v>
       </c>
       <c r="E2" t="n">
-        <v>44191</v>
+        <v>410063</v>
       </c>
       <c r="F2" t="n">
-        <v>54993</v>
+        <v>563327</v>
       </c>
       <c r="G2" t="n">
-        <v>80596</v>
+        <v>148750</v>
       </c>
       <c r="H2" t="n">
-        <v>20815</v>
+        <v>620991</v>
       </c>
       <c r="I2" t="n">
-        <v>97301</v>
+        <v>209170</v>
       </c>
       <c r="J2" t="n">
-        <v>44675</v>
+        <v>245528</v>
       </c>
       <c r="K2" t="n">
-        <v>114261</v>
+        <v>396064</v>
       </c>
       <c r="L2" t="n">
-        <v>5065</v>
+        <v>513902</v>
       </c>
       <c r="M2" t="n">
-        <v>97492</v>
+        <v>647598</v>
       </c>
       <c r="N2" t="n">
-        <v>82203</v>
+        <v>565839</v>
       </c>
       <c r="O2" t="n">
-        <v>93985</v>
+        <v>305917</v>
       </c>
       <c r="P2" t="n">
-        <v>49063</v>
+        <v>41749</v>
       </c>
       <c r="Q2" t="n">
-        <v>47242</v>
+        <v>742</v>
       </c>
       <c r="R2" t="n">
-        <v>10631</v>
+        <v>265974</v>
       </c>
       <c r="S2" t="n">
-        <v>28389</v>
+        <v>362816</v>
       </c>
       <c r="T2" t="n">
-        <v>65955</v>
+        <v>5069</v>
       </c>
       <c r="U2" t="n">
-        <v>20619</v>
+        <v>347608</v>
       </c>
       <c r="V2" t="n">
-        <v>124725</v>
+        <v>163580</v>
       </c>
       <c r="W2" t="n">
-        <v>24543</v>
+        <v>299077</v>
       </c>
       <c r="X2" t="n">
+        <v>9352</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>567345</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>47944</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>385573</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>200505</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>40689</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>684802</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>738042</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>659136</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>298046</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>10107</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>90224</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>61636</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>316822</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>485412</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>546092</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>746598</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>20170</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>707552</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>331428</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>798602</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>333388</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>444425</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>766749</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>26571</v>
+      </c>
+      <c r="AW2" t="n">
+        <v>174125</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>455547</v>
+      </c>
+      <c r="AY2" t="n">
         <v>0</v>
       </c>
-      <c r="Y2" t="n">
-        <v>62541</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>10961</v>
-      </c>
-      <c r="AA2" t="n">
-        <v>87159</v>
-      </c>
-      <c r="AB2" t="n">
-        <v>865</v>
-      </c>
-      <c r="AC2" t="n">
-        <v>53599</v>
-      </c>
-      <c r="AD2" t="n">
-        <v>126</v>
-      </c>
-      <c r="AE2" t="n">
-        <v>59744</v>
-      </c>
-      <c r="AF2" t="n">
-        <v>126355</v>
-      </c>
-      <c r="AG2" t="n">
-        <v>76232</v>
-      </c>
-      <c r="AH2" t="n">
-        <v>66149</v>
-      </c>
-      <c r="AI2" t="n">
-        <v>93134</v>
-      </c>
-      <c r="AJ2" t="n">
-        <v>74327</v>
-      </c>
-      <c r="AK2" t="n">
-        <v>63316</v>
-      </c>
-      <c r="AL2" t="n">
-        <v>119564</v>
-      </c>
-      <c r="AM2" t="n">
-        <v>89070</v>
-      </c>
-      <c r="AN2" t="n">
-        <v>100908</v>
-      </c>
-      <c r="AO2" t="n">
-        <v>70978</v>
-      </c>
-      <c r="AP2" t="n">
-        <v>28379</v>
-      </c>
-      <c r="AQ2" t="n">
-        <v>78993</v>
-      </c>
-      <c r="AR2" t="n">
-        <v>84607</v>
-      </c>
-      <c r="AS2" t="n">
-        <v>98471</v>
-      </c>
-      <c r="AT2" t="n">
-        <v>103129</v>
-      </c>
-      <c r="AU2" t="n">
-        <v>107829</v>
-      </c>
-      <c r="AV2" t="n">
-        <v>93107</v>
-      </c>
-      <c r="AW2" t="n">
-        <v>66967</v>
-      </c>
-      <c r="AX2" t="n">
-        <v>59474</v>
-      </c>
-      <c r="AY2" t="n">
-        <v>38913</v>
-      </c>
       <c r="AZ2" t="n">
-        <v>5642</v>
+        <v>83135</v>
       </c>
       <c r="BA2" t="n">
-        <v>120143</v>
+        <v>779207</v>
       </c>
       <c r="BB2" t="n">
-        <v>35039</v>
+        <v>762998</v>
       </c>
       <c r="BC2" t="n">
-        <v>116512</v>
+        <v>412537</v>
       </c>
       <c r="BD2" t="n">
-        <v>25749</v>
+        <v>674046</v>
       </c>
       <c r="BE2" t="n">
-        <v>28506</v>
+        <v>749533</v>
       </c>
       <c r="BF2" t="n">
-        <v>72483</v>
+        <v>381121</v>
       </c>
       <c r="BG2" t="n">
-        <v>13784</v>
+        <v>126203</v>
       </c>
       <c r="BH2" t="n">
-        <v>41752</v>
+        <v>509335</v>
       </c>
       <c r="BI2" t="n">
-        <v>28947</v>
+        <v>650448</v>
       </c>
       <c r="BJ2" t="n">
-        <v>16433</v>
+        <v>292037</v>
       </c>
       <c r="BK2" t="n">
-        <v>16481</v>
+        <v>443827</v>
       </c>
       <c r="BL2" t="n">
-        <v>49973</v>
+        <v>454506</v>
       </c>
       <c r="BM2" t="n">
-        <v>107018</v>
+        <v>518512</v>
       </c>
       <c r="BN2" t="n">
-        <v>35814</v>
+        <v>52837</v>
       </c>
       <c r="BO2" t="n">
-        <v>20030</v>
+        <v>140135</v>
       </c>
       <c r="BP2" t="n">
-        <v>38728</v>
+        <v>275668</v>
       </c>
       <c r="BQ2" t="n">
-        <v>30624</v>
+        <v>489616</v>
       </c>
       <c r="BR2" t="n">
-        <v>6052</v>
+        <v>755474</v>
       </c>
       <c r="BS2" t="n">
-        <v>121882</v>
+        <v>218021</v>
       </c>
       <c r="BT2" t="n">
-        <v>42103</v>
+        <v>622775</v>
       </c>
       <c r="BU2" t="n">
-        <v>24950</v>
+        <v>251454</v>
       </c>
       <c r="BV2" t="n">
-        <v>115799</v>
+        <v>145564</v>
       </c>
       <c r="BW2" t="n">
-        <v>15994</v>
+        <v>188145</v>
       </c>
       <c r="BX2" t="n">
-        <v>45938</v>
+        <v>673569</v>
       </c>
       <c r="BY2" t="n">
-        <v>87813</v>
+        <v>722758</v>
       </c>
       <c r="BZ2" t="n">
-        <v>6680</v>
+        <v>336321</v>
       </c>
       <c r="CA2" t="n">
-        <v>459</v>
+        <v>564576</v>
       </c>
       <c r="CB2" t="n">
-        <v>12877</v>
+        <v>528812</v>
       </c>
       <c r="CC2" t="n">
-        <v>86093</v>
+        <v>111220</v>
       </c>
       <c r="CD2" t="n">
-        <v>64985</v>
+        <v>265007</v>
       </c>
       <c r="CE2" t="n">
-        <v>111461</v>
+        <v>425101</v>
       </c>
       <c r="CF2" t="n">
-        <v>58149</v>
+        <v>356587</v>
       </c>
       <c r="CG2" t="n">
-        <v>9455</v>
+        <v>827560</v>
       </c>
       <c r="CH2" t="n">
-        <v>19337</v>
+        <v>226058</v>
       </c>
       <c r="CI2" t="n">
-        <v>83255</v>
+        <v>113282</v>
       </c>
       <c r="CJ2" t="n">
-        <v>113044</v>
+        <v>394212</v>
       </c>
       <c r="CK2" t="n">
-        <v>39530</v>
+        <v>162065</v>
       </c>
       <c r="CL2" t="n">
-        <v>2889</v>
+        <v>595300</v>
       </c>
       <c r="CM2" t="n">
-        <v>77648</v>
+        <v>104858</v>
       </c>
       <c r="CN2" t="n">
-        <v>57372</v>
+        <v>117416</v>
       </c>
       <c r="CO2" t="n">
-        <v>105456</v>
+        <v>697334</v>
       </c>
       <c r="CP2" t="n">
-        <v>81409</v>
+        <v>789881</v>
       </c>
       <c r="CQ2" t="n">
-        <v>108994</v>
+        <v>815861</v>
       </c>
       <c r="CR2" t="n">
-        <v>49638</v>
+        <v>200012</v>
       </c>
       <c r="CS2" t="n">
-        <v>33110</v>
+        <v>446426</v>
       </c>
       <c r="CT2" t="n">
-        <v>10341</v>
+        <v>66400</v>
       </c>
       <c r="CU2" t="n">
-        <v>22740</v>
+        <v>586946</v>
       </c>
       <c r="CV2" t="n">
-        <v>91812</v>
+        <v>467396</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new run of brkga
</commit_message>
<xml_diff>
--- a/code/resultados/NWJSSP_OADG_BRKGA.xlsx
+++ b/code/resultados/NWJSSP_OADG_BRKGA.xlsx
@@ -432,7 +432,7 @@
         <v>308</v>
       </c>
       <c r="B1" t="n">
-        <v>3226</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="2">
@@ -471,312 +471,312 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>6244284</v>
+        <v>6449398</v>
       </c>
       <c r="B1" t="n">
-        <v>3614722</v>
+        <v>3607158</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>33729</v>
+        <v>3627</v>
       </c>
       <c r="B2" t="n">
-        <v>53695</v>
+        <v>97214</v>
       </c>
       <c r="C2" t="n">
-        <v>70605</v>
+        <v>9967</v>
       </c>
       <c r="D2" t="n">
-        <v>48865</v>
+        <v>118127</v>
       </c>
       <c r="E2" t="n">
-        <v>44191</v>
+        <v>64059</v>
       </c>
       <c r="F2" t="n">
-        <v>54993</v>
+        <v>119936</v>
       </c>
       <c r="G2" t="n">
-        <v>80596</v>
+        <v>118677</v>
       </c>
       <c r="H2" t="n">
-        <v>20815</v>
+        <v>30082</v>
       </c>
       <c r="I2" t="n">
-        <v>97301</v>
+        <v>60105</v>
       </c>
       <c r="J2" t="n">
-        <v>44675</v>
+        <v>85975</v>
       </c>
       <c r="K2" t="n">
-        <v>114261</v>
+        <v>49726</v>
       </c>
       <c r="L2" t="n">
-        <v>5065</v>
+        <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>97492</v>
+        <v>34536</v>
       </c>
       <c r="N2" t="n">
-        <v>82203</v>
+        <v>13836</v>
       </c>
       <c r="O2" t="n">
-        <v>93985</v>
+        <v>75027</v>
       </c>
       <c r="P2" t="n">
-        <v>49063</v>
+        <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>47242</v>
+        <v>13854</v>
       </c>
       <c r="R2" t="n">
-        <v>10631</v>
+        <v>72731</v>
       </c>
       <c r="S2" t="n">
-        <v>28389</v>
+        <v>108710</v>
       </c>
       <c r="T2" t="n">
-        <v>65955</v>
+        <v>103462</v>
       </c>
       <c r="U2" t="n">
-        <v>20619</v>
+        <v>107503</v>
       </c>
       <c r="V2" t="n">
-        <v>124725</v>
+        <v>34465</v>
       </c>
       <c r="W2" t="n">
-        <v>24543</v>
+        <v>81865</v>
       </c>
       <c r="X2" t="n">
-        <v>0</v>
+        <v>90262</v>
       </c>
       <c r="Y2" t="n">
-        <v>62541</v>
+        <v>104278</v>
       </c>
       <c r="Z2" t="n">
-        <v>10961</v>
+        <v>27454</v>
       </c>
       <c r="AA2" t="n">
-        <v>87159</v>
+        <v>56310</v>
       </c>
       <c r="AB2" t="n">
-        <v>865</v>
+        <v>83518</v>
       </c>
       <c r="AC2" t="n">
-        <v>53599</v>
+        <v>33670</v>
       </c>
       <c r="AD2" t="n">
-        <v>126</v>
+        <v>103981</v>
       </c>
       <c r="AE2" t="n">
-        <v>59744</v>
+        <v>53445</v>
       </c>
       <c r="AF2" t="n">
-        <v>126355</v>
+        <v>67696</v>
       </c>
       <c r="AG2" t="n">
-        <v>76232</v>
+        <v>48579</v>
       </c>
       <c r="AH2" t="n">
-        <v>66149</v>
+        <v>17108</v>
       </c>
       <c r="AI2" t="n">
-        <v>93134</v>
+        <v>75884</v>
       </c>
       <c r="AJ2" t="n">
-        <v>74327</v>
+        <v>43711</v>
       </c>
       <c r="AK2" t="n">
-        <v>63316</v>
+        <v>99520</v>
       </c>
       <c r="AL2" t="n">
-        <v>119564</v>
+        <v>21074</v>
       </c>
       <c r="AM2" t="n">
-        <v>89070</v>
+        <v>127286</v>
       </c>
       <c r="AN2" t="n">
-        <v>100908</v>
+        <v>111403</v>
       </c>
       <c r="AO2" t="n">
-        <v>70978</v>
+        <v>123699</v>
       </c>
       <c r="AP2" t="n">
-        <v>28379</v>
+        <v>4192</v>
       </c>
       <c r="AQ2" t="n">
-        <v>78993</v>
+        <v>78966</v>
       </c>
       <c r="AR2" t="n">
-        <v>84607</v>
+        <v>74177</v>
       </c>
       <c r="AS2" t="n">
-        <v>98471</v>
+        <v>10183</v>
       </c>
       <c r="AT2" t="n">
-        <v>103129</v>
+        <v>87849</v>
       </c>
       <c r="AU2" t="n">
-        <v>107829</v>
+        <v>98331</v>
       </c>
       <c r="AV2" t="n">
-        <v>93107</v>
+        <v>18803</v>
       </c>
       <c r="AW2" t="n">
-        <v>66967</v>
+        <v>44008</v>
       </c>
       <c r="AX2" t="n">
-        <v>59474</v>
+        <v>77670</v>
       </c>
       <c r="AY2" t="n">
-        <v>38913</v>
+        <v>60827</v>
       </c>
       <c r="AZ2" t="n">
-        <v>5642</v>
+        <v>28128</v>
       </c>
       <c r="BA2" t="n">
-        <v>120143</v>
+        <v>84384</v>
       </c>
       <c r="BB2" t="n">
-        <v>35039</v>
+        <v>89444</v>
       </c>
       <c r="BC2" t="n">
-        <v>116512</v>
+        <v>66241</v>
       </c>
       <c r="BD2" t="n">
-        <v>25749</v>
+        <v>64200</v>
       </c>
       <c r="BE2" t="n">
-        <v>28506</v>
+        <v>49569</v>
       </c>
       <c r="BF2" t="n">
-        <v>72483</v>
+        <v>124472</v>
       </c>
       <c r="BG2" t="n">
-        <v>13784</v>
+        <v>72197</v>
       </c>
       <c r="BH2" t="n">
-        <v>41752</v>
+        <v>113749</v>
       </c>
       <c r="BI2" t="n">
-        <v>28947</v>
+        <v>56617</v>
       </c>
       <c r="BJ2" t="n">
-        <v>16433</v>
+        <v>8745</v>
       </c>
       <c r="BK2" t="n">
-        <v>16481</v>
+        <v>105572</v>
       </c>
       <c r="BL2" t="n">
-        <v>49973</v>
+        <v>25844</v>
       </c>
       <c r="BM2" t="n">
-        <v>107018</v>
+        <v>89864</v>
       </c>
       <c r="BN2" t="n">
-        <v>35814</v>
+        <v>4023</v>
       </c>
       <c r="BO2" t="n">
-        <v>20030</v>
+        <v>3977</v>
       </c>
       <c r="BP2" t="n">
-        <v>38728</v>
+        <v>60319</v>
       </c>
       <c r="BQ2" t="n">
-        <v>30624</v>
+        <v>38366</v>
       </c>
       <c r="BR2" t="n">
-        <v>6052</v>
+        <v>8911</v>
       </c>
       <c r="BS2" t="n">
-        <v>121882</v>
+        <v>115972</v>
       </c>
       <c r="BT2" t="n">
-        <v>42103</v>
+        <v>81186</v>
       </c>
       <c r="BU2" t="n">
-        <v>24950</v>
+        <v>22479</v>
       </c>
       <c r="BV2" t="n">
-        <v>115799</v>
+        <v>43809</v>
       </c>
       <c r="BW2" t="n">
-        <v>15994</v>
+        <v>33039</v>
       </c>
       <c r="BX2" t="n">
-        <v>45938</v>
+        <v>29366</v>
       </c>
       <c r="BY2" t="n">
-        <v>87813</v>
+        <v>109404</v>
       </c>
       <c r="BZ2" t="n">
-        <v>6680</v>
+        <v>44873</v>
       </c>
       <c r="CA2" t="n">
-        <v>459</v>
+        <v>24117</v>
       </c>
       <c r="CB2" t="n">
-        <v>12877</v>
+        <v>94118</v>
       </c>
       <c r="CC2" t="n">
-        <v>86093</v>
+        <v>52640</v>
       </c>
       <c r="CD2" t="n">
-        <v>64985</v>
+        <v>39828</v>
       </c>
       <c r="CE2" t="n">
-        <v>111461</v>
+        <v>37632</v>
       </c>
       <c r="CF2" t="n">
-        <v>58149</v>
+        <v>41507</v>
       </c>
       <c r="CG2" t="n">
-        <v>9455</v>
+        <v>92237</v>
       </c>
       <c r="CH2" t="n">
-        <v>19337</v>
+        <v>96310</v>
       </c>
       <c r="CI2" t="n">
-        <v>83255</v>
+        <v>93109</v>
       </c>
       <c r="CJ2" t="n">
-        <v>113044</v>
+        <v>31040</v>
       </c>
       <c r="CK2" t="n">
-        <v>39530</v>
+        <v>106369</v>
       </c>
       <c r="CL2" t="n">
-        <v>2889</v>
+        <v>14862</v>
       </c>
       <c r="CM2" t="n">
-        <v>77648</v>
+        <v>20282</v>
       </c>
       <c r="CN2" t="n">
-        <v>57372</v>
+        <v>11884</v>
       </c>
       <c r="CO2" t="n">
-        <v>105456</v>
+        <v>53266</v>
       </c>
       <c r="CP2" t="n">
-        <v>81409</v>
+        <v>83</v>
       </c>
       <c r="CQ2" t="n">
-        <v>108994</v>
+        <v>99719</v>
       </c>
       <c r="CR2" t="n">
-        <v>49638</v>
+        <v>15015</v>
       </c>
       <c r="CS2" t="n">
-        <v>33110</v>
+        <v>70285</v>
       </c>
       <c r="CT2" t="n">
-        <v>10341</v>
+        <v>48705</v>
       </c>
       <c r="CU2" t="n">
-        <v>22740</v>
+        <v>55928</v>
       </c>
       <c r="CV2" t="n">
-        <v>91812</v>
+        <v>23518</v>
       </c>
     </row>
   </sheetData>
@@ -795,312 +795,312 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>43470943</v>
+        <v>43832744</v>
       </c>
       <c r="B1" t="n">
-        <v>4577840</v>
+        <v>4347283</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>616769</v>
+        <v>810612</v>
       </c>
       <c r="B2" t="n">
-        <v>701676</v>
+        <v>589691</v>
       </c>
       <c r="C2" t="n">
-        <v>105574</v>
+        <v>188880</v>
       </c>
       <c r="D2" t="n">
-        <v>63797</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>318151</v>
+        <v>484107</v>
       </c>
       <c r="F2" t="n">
-        <v>181590</v>
+        <v>187999</v>
       </c>
       <c r="G2" t="n">
-        <v>673373</v>
+        <v>671387</v>
       </c>
       <c r="H2" t="n">
-        <v>450641</v>
+        <v>433594</v>
       </c>
       <c r="I2" t="n">
-        <v>248670</v>
+        <v>655929</v>
       </c>
       <c r="J2" t="n">
-        <v>742073</v>
+        <v>409677</v>
       </c>
       <c r="K2" t="n">
-        <v>519730</v>
+        <v>39224</v>
       </c>
       <c r="L2" t="n">
-        <v>502030</v>
+        <v>601148</v>
       </c>
       <c r="M2" t="n">
-        <v>749100</v>
+        <v>483973</v>
       </c>
       <c r="N2" t="n">
-        <v>465421</v>
+        <v>373075</v>
       </c>
       <c r="O2" t="n">
-        <v>485204</v>
+        <v>47431</v>
       </c>
       <c r="P2" t="n">
-        <v>38928</v>
+        <v>834295</v>
       </c>
       <c r="Q2" t="n">
-        <v>23327</v>
+        <v>619528</v>
       </c>
       <c r="R2" t="n">
-        <v>326696</v>
+        <v>308010</v>
       </c>
       <c r="S2" t="n">
-        <v>600466</v>
+        <v>278675</v>
       </c>
       <c r="T2" t="n">
-        <v>729950</v>
+        <v>635525</v>
       </c>
       <c r="U2" t="n">
-        <v>0</v>
+        <v>1074</v>
       </c>
       <c r="V2" t="n">
-        <v>634600</v>
+        <v>423317</v>
       </c>
       <c r="W2" t="n">
-        <v>615790</v>
+        <v>689530</v>
       </c>
       <c r="X2" t="n">
-        <v>85681</v>
+        <v>315118</v>
       </c>
       <c r="Y2" t="n">
-        <v>922</v>
+        <v>739628</v>
       </c>
       <c r="Z2" t="n">
-        <v>784078</v>
+        <v>63872</v>
       </c>
       <c r="AA2" t="n">
-        <v>413607</v>
+        <v>107501</v>
       </c>
       <c r="AB2" t="n">
-        <v>147942</v>
+        <v>294100</v>
       </c>
       <c r="AC2" t="n">
-        <v>53386</v>
+        <v>651444</v>
       </c>
       <c r="AD2" t="n">
-        <v>761058</v>
+        <v>484832</v>
       </c>
       <c r="AE2" t="n">
-        <v>675764</v>
+        <v>688879</v>
       </c>
       <c r="AF2" t="n">
-        <v>379713</v>
+        <v>777081</v>
       </c>
       <c r="AG2" t="n">
-        <v>785522</v>
+        <v>256601</v>
       </c>
       <c r="AH2" t="n">
-        <v>519424</v>
+        <v>209325</v>
       </c>
       <c r="AI2" t="n">
-        <v>760036</v>
+        <v>9883</v>
       </c>
       <c r="AJ2" t="n">
-        <v>740832</v>
+        <v>279825</v>
       </c>
       <c r="AK2" t="n">
-        <v>566812</v>
+        <v>151432</v>
       </c>
       <c r="AL2" t="n">
-        <v>28179</v>
+        <v>451107</v>
       </c>
       <c r="AM2" t="n">
-        <v>305152</v>
+        <v>632932</v>
       </c>
       <c r="AN2" t="n">
-        <v>646807</v>
+        <v>345564</v>
       </c>
       <c r="AO2" t="n">
-        <v>654480</v>
+        <v>316603</v>
       </c>
       <c r="AP2" t="n">
-        <v>557919</v>
+        <v>81370</v>
       </c>
       <c r="AQ2" t="n">
-        <v>402954</v>
+        <v>236252</v>
       </c>
       <c r="AR2" t="n">
-        <v>219769</v>
+        <v>578140</v>
       </c>
       <c r="AS2" t="n">
-        <v>71471</v>
+        <v>751172</v>
       </c>
       <c r="AT2" t="n">
-        <v>559134</v>
+        <v>261091</v>
       </c>
       <c r="AU2" t="n">
-        <v>215606</v>
+        <v>692397</v>
       </c>
       <c r="AV2" t="n">
-        <v>226577</v>
+        <v>411252</v>
       </c>
       <c r="AW2" t="n">
-        <v>10537</v>
+        <v>546197</v>
       </c>
       <c r="AX2" t="n">
-        <v>787550</v>
+        <v>228875</v>
       </c>
       <c r="AY2" t="n">
-        <v>160932</v>
+        <v>490723</v>
       </c>
       <c r="AZ2" t="n">
-        <v>25139</v>
+        <v>80871</v>
       </c>
       <c r="BA2" t="n">
-        <v>171556</v>
+        <v>360197</v>
       </c>
       <c r="BB2" t="n">
-        <v>463072</v>
+        <v>470203</v>
       </c>
       <c r="BC2" t="n">
-        <v>496202</v>
+        <v>460996</v>
       </c>
       <c r="BD2" t="n">
-        <v>534523</v>
+        <v>351249</v>
       </c>
       <c r="BE2" t="n">
-        <v>365686</v>
+        <v>721273</v>
       </c>
       <c r="BF2" t="n">
-        <v>282981</v>
+        <v>508710</v>
       </c>
       <c r="BG2" t="n">
-        <v>386227</v>
+        <v>803707</v>
       </c>
       <c r="BH2" t="n">
-        <v>262079</v>
+        <v>84407</v>
       </c>
       <c r="BI2" t="n">
-        <v>584793</v>
+        <v>763510</v>
       </c>
       <c r="BJ2" t="n">
-        <v>562231</v>
+        <v>6976</v>
       </c>
       <c r="BK2" t="n">
-        <v>80504</v>
+        <v>616242</v>
       </c>
       <c r="BL2" t="n">
-        <v>204873</v>
+        <v>576653</v>
       </c>
       <c r="BM2" t="n">
-        <v>336453</v>
+        <v>536105</v>
       </c>
       <c r="BN2" t="n">
-        <v>237183</v>
+        <v>26264</v>
       </c>
       <c r="BO2" t="n">
-        <v>131331</v>
+        <v>441908</v>
       </c>
       <c r="BP2" t="n">
-        <v>493925</v>
+        <v>9474</v>
       </c>
       <c r="BQ2" t="n">
-        <v>112644</v>
+        <v>709524</v>
       </c>
       <c r="BR2" t="n">
-        <v>588187</v>
+        <v>125511</v>
       </c>
       <c r="BS2" t="n">
-        <v>539337</v>
+        <v>335590</v>
       </c>
       <c r="BT2" t="n">
-        <v>353666</v>
+        <v>545590</v>
       </c>
       <c r="BU2" t="n">
-        <v>418829</v>
+        <v>73726</v>
       </c>
       <c r="BV2" t="n">
-        <v>701741</v>
+        <v>822065</v>
       </c>
       <c r="BW2" t="n">
-        <v>402149</v>
+        <v>385159</v>
       </c>
       <c r="BX2" t="n">
-        <v>453534</v>
+        <v>364275</v>
       </c>
       <c r="BY2" t="n">
-        <v>294413</v>
+        <v>41804</v>
       </c>
       <c r="BZ2" t="n">
-        <v>103082</v>
+        <v>423091</v>
       </c>
       <c r="CA2" t="n">
-        <v>387288</v>
+        <v>83462</v>
       </c>
       <c r="CB2" t="n">
-        <v>819588</v>
+        <v>715036</v>
       </c>
       <c r="CC2" t="n">
-        <v>350158</v>
+        <v>175029</v>
       </c>
       <c r="CD2" t="n">
-        <v>127203</v>
+        <v>242884</v>
       </c>
       <c r="CE2" t="n">
-        <v>420036</v>
+        <v>133626</v>
       </c>
       <c r="CF2" t="n">
-        <v>279940</v>
+        <v>243797</v>
       </c>
       <c r="CG2" t="n">
-        <v>159376</v>
+        <v>185404</v>
       </c>
       <c r="CH2" t="n">
-        <v>3576</v>
+        <v>546580</v>
       </c>
       <c r="CI2" t="n">
-        <v>102261</v>
+        <v>791408</v>
       </c>
       <c r="CJ2" t="n">
-        <v>161264</v>
+        <v>205160</v>
       </c>
       <c r="CK2" t="n">
-        <v>434412</v>
+        <v>518643</v>
       </c>
       <c r="CL2" t="n">
-        <v>187678</v>
+        <v>746960</v>
       </c>
       <c r="CM2" t="n">
-        <v>487016</v>
+        <v>124092</v>
       </c>
       <c r="CN2" t="n">
-        <v>268026</v>
+        <v>373494</v>
       </c>
       <c r="CO2" t="n">
-        <v>353998</v>
+        <v>392468</v>
       </c>
       <c r="CP2" t="n">
-        <v>738027</v>
+        <v>114643</v>
       </c>
       <c r="CQ2" t="n">
-        <v>308644</v>
+        <v>161604</v>
       </c>
       <c r="CR2" t="n">
-        <v>133158</v>
+        <v>161658</v>
       </c>
       <c r="CS2" t="n">
-        <v>199337</v>
+        <v>216050</v>
       </c>
       <c r="CT2" t="n">
-        <v>708015</v>
+        <v>114267</v>
       </c>
       <c r="CU2" t="n">
-        <v>695233</v>
+        <v>290441</v>
       </c>
       <c r="CV2" t="n">
-        <v>246301</v>
+        <v>832413</v>
       </c>
     </row>
   </sheetData>
@@ -1119,10 +1119,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>44086748</v>
+        <v>44410066</v>
       </c>
       <c r="B1" t="n">
-        <v>4498508</v>
+        <v>3701068</v>
       </c>
       <c r="C1" t="inlineStr"/>
       <c r="D1" t="inlineStr"/>
@@ -1225,304 +1225,304 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>608588</v>
+        <v>133008</v>
       </c>
       <c r="B2" t="n">
-        <v>818806</v>
+        <v>439060</v>
       </c>
       <c r="C2" t="n">
-        <v>542197</v>
+        <v>667799</v>
       </c>
       <c r="D2" t="n">
-        <v>485751</v>
+        <v>448069</v>
       </c>
       <c r="E2" t="n">
-        <v>410063</v>
+        <v>719787</v>
       </c>
       <c r="F2" t="n">
-        <v>563327</v>
+        <v>815160</v>
       </c>
       <c r="G2" t="n">
-        <v>148750</v>
+        <v>201045</v>
       </c>
       <c r="H2" t="n">
-        <v>620991</v>
+        <v>403257</v>
       </c>
       <c r="I2" t="n">
-        <v>209170</v>
+        <v>326147</v>
       </c>
       <c r="J2" t="n">
-        <v>245528</v>
+        <v>526052</v>
       </c>
       <c r="K2" t="n">
-        <v>396064</v>
+        <v>840963</v>
       </c>
       <c r="L2" t="n">
-        <v>513902</v>
+        <v>667276</v>
       </c>
       <c r="M2" t="n">
-        <v>647598</v>
+        <v>693101</v>
       </c>
       <c r="N2" t="n">
-        <v>565839</v>
+        <v>98087</v>
       </c>
       <c r="O2" t="n">
-        <v>305917</v>
+        <v>760415</v>
       </c>
       <c r="P2" t="n">
-        <v>41749</v>
+        <v>601338</v>
       </c>
       <c r="Q2" t="n">
-        <v>742</v>
+        <v>163926</v>
       </c>
       <c r="R2" t="n">
-        <v>265974</v>
+        <v>214712</v>
       </c>
       <c r="S2" t="n">
-        <v>362816</v>
+        <v>632787</v>
       </c>
       <c r="T2" t="n">
-        <v>5069</v>
+        <v>643385</v>
       </c>
       <c r="U2" t="n">
-        <v>347608</v>
+        <v>513452</v>
       </c>
       <c r="V2" t="n">
-        <v>163580</v>
+        <v>465270</v>
       </c>
       <c r="W2" t="n">
-        <v>299077</v>
+        <v>428919</v>
       </c>
       <c r="X2" t="n">
-        <v>9352</v>
+        <v>678805</v>
       </c>
       <c r="Y2" t="n">
-        <v>567345</v>
+        <v>2161</v>
       </c>
       <c r="Z2" t="n">
-        <v>47944</v>
+        <v>482657</v>
       </c>
       <c r="AA2" t="n">
-        <v>385573</v>
+        <v>289974</v>
       </c>
       <c r="AB2" t="n">
-        <v>200505</v>
+        <v>353800</v>
       </c>
       <c r="AC2" t="n">
-        <v>40689</v>
+        <v>150060</v>
       </c>
       <c r="AD2" t="n">
-        <v>684802</v>
+        <v>523528</v>
       </c>
       <c r="AE2" t="n">
-        <v>738042</v>
+        <v>93503</v>
       </c>
       <c r="AF2" t="n">
-        <v>659136</v>
+        <v>133201</v>
       </c>
       <c r="AG2" t="n">
-        <v>298046</v>
+        <v>360389</v>
       </c>
       <c r="AH2" t="n">
-        <v>10107</v>
+        <v>69987</v>
       </c>
       <c r="AI2" t="n">
-        <v>90224</v>
+        <v>479069</v>
       </c>
       <c r="AJ2" t="n">
-        <v>61636</v>
+        <v>784952</v>
       </c>
       <c r="AK2" t="n">
-        <v>316822</v>
+        <v>840287</v>
       </c>
       <c r="AL2" t="n">
-        <v>485412</v>
+        <v>37155</v>
       </c>
       <c r="AM2" t="n">
-        <v>546092</v>
+        <v>238228</v>
       </c>
       <c r="AN2" t="n">
-        <v>746598</v>
+        <v>163641</v>
       </c>
       <c r="AO2" t="n">
-        <v>20170</v>
+        <v>376592</v>
       </c>
       <c r="AP2" t="n">
-        <v>707552</v>
+        <v>691090</v>
       </c>
       <c r="AQ2" t="n">
-        <v>331428</v>
+        <v>367331</v>
       </c>
       <c r="AR2" t="n">
-        <v>798602</v>
+        <v>138787</v>
       </c>
       <c r="AS2" t="n">
-        <v>333388</v>
+        <v>728569</v>
       </c>
       <c r="AT2" t="n">
-        <v>444425</v>
+        <v>410743</v>
       </c>
       <c r="AU2" t="n">
-        <v>766749</v>
+        <v>56507</v>
       </c>
       <c r="AV2" t="n">
-        <v>26571</v>
+        <v>2438</v>
       </c>
       <c r="AW2" t="n">
-        <v>174125</v>
+        <v>556634</v>
       </c>
       <c r="AX2" t="n">
-        <v>455547</v>
+        <v>624930</v>
       </c>
       <c r="AY2" t="n">
+        <v>770341</v>
+      </c>
+      <c r="AZ2" t="n">
+        <v>16914</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>76356</v>
+      </c>
+      <c r="BB2" t="n">
+        <v>249605</v>
+      </c>
+      <c r="BC2" t="n">
+        <v>57243</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>601895</v>
+      </c>
+      <c r="BE2" t="n">
+        <v>42095</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>589515</v>
+      </c>
+      <c r="BG2" t="n">
+        <v>503682</v>
+      </c>
+      <c r="BH2" t="n">
+        <v>419360</v>
+      </c>
+      <c r="BI2" t="n">
+        <v>288893</v>
+      </c>
+      <c r="BJ2" t="n">
+        <v>574071</v>
+      </c>
+      <c r="BK2" t="n">
+        <v>748939</v>
+      </c>
+      <c r="BL2" t="n">
+        <v>487643</v>
+      </c>
+      <c r="BM2" t="n">
+        <v>222256</v>
+      </c>
+      <c r="BN2" t="n">
+        <v>76099</v>
+      </c>
+      <c r="BO2" t="n">
+        <v>805972</v>
+      </c>
+      <c r="BP2" t="n">
+        <v>261988</v>
+      </c>
+      <c r="BQ2" t="n">
+        <v>191458</v>
+      </c>
+      <c r="BR2" t="n">
+        <v>837637</v>
+      </c>
+      <c r="BS2" t="n">
+        <v>631999</v>
+      </c>
+      <c r="BT2" t="n">
+        <v>317034</v>
+      </c>
+      <c r="BU2" t="n">
+        <v>798074</v>
+      </c>
+      <c r="BV2" t="n">
+        <v>59319</v>
+      </c>
+      <c r="BW2" t="n">
+        <v>340174</v>
+      </c>
+      <c r="BX2" t="n">
+        <v>206992</v>
+      </c>
+      <c r="BY2" t="n">
+        <v>138697</v>
+      </c>
+      <c r="BZ2" t="n">
+        <v>17732</v>
+      </c>
+      <c r="CA2" t="n">
+        <v>306748</v>
+      </c>
+      <c r="CB2" t="n">
+        <v>350973</v>
+      </c>
+      <c r="CC2" t="n">
+        <v>714811</v>
+      </c>
+      <c r="CD2" t="n">
+        <v>251652</v>
+      </c>
+      <c r="CE2" t="n">
         <v>0</v>
       </c>
-      <c r="AZ2" t="n">
-        <v>83135</v>
-      </c>
-      <c r="BA2" t="n">
-        <v>779207</v>
-      </c>
-      <c r="BB2" t="n">
-        <v>762998</v>
-      </c>
-      <c r="BC2" t="n">
-        <v>412537</v>
-      </c>
-      <c r="BD2" t="n">
-        <v>674046</v>
-      </c>
-      <c r="BE2" t="n">
-        <v>749533</v>
-      </c>
-      <c r="BF2" t="n">
-        <v>381121</v>
-      </c>
-      <c r="BG2" t="n">
-        <v>126203</v>
-      </c>
-      <c r="BH2" t="n">
-        <v>509335</v>
-      </c>
-      <c r="BI2" t="n">
-        <v>650448</v>
-      </c>
-      <c r="BJ2" t="n">
-        <v>292037</v>
-      </c>
-      <c r="BK2" t="n">
-        <v>443827</v>
-      </c>
-      <c r="BL2" t="n">
-        <v>454506</v>
-      </c>
-      <c r="BM2" t="n">
-        <v>518512</v>
-      </c>
-      <c r="BN2" t="n">
-        <v>52837</v>
-      </c>
-      <c r="BO2" t="n">
-        <v>140135</v>
-      </c>
-      <c r="BP2" t="n">
-        <v>275668</v>
-      </c>
-      <c r="BQ2" t="n">
-        <v>489616</v>
-      </c>
-      <c r="BR2" t="n">
-        <v>755474</v>
-      </c>
-      <c r="BS2" t="n">
-        <v>218021</v>
-      </c>
-      <c r="BT2" t="n">
-        <v>622775</v>
-      </c>
-      <c r="BU2" t="n">
-        <v>251454</v>
-      </c>
-      <c r="BV2" t="n">
-        <v>145564</v>
-      </c>
-      <c r="BW2" t="n">
-        <v>188145</v>
-      </c>
-      <c r="BX2" t="n">
-        <v>673569</v>
-      </c>
-      <c r="BY2" t="n">
-        <v>722758</v>
-      </c>
-      <c r="BZ2" t="n">
-        <v>336321</v>
-      </c>
-      <c r="CA2" t="n">
-        <v>564576</v>
-      </c>
-      <c r="CB2" t="n">
-        <v>528812</v>
-      </c>
-      <c r="CC2" t="n">
-        <v>111220</v>
-      </c>
-      <c r="CD2" t="n">
-        <v>265007</v>
-      </c>
-      <c r="CE2" t="n">
-        <v>425101</v>
-      </c>
       <c r="CF2" t="n">
-        <v>356587</v>
+        <v>267148</v>
       </c>
       <c r="CG2" t="n">
-        <v>827560</v>
+        <v>130088</v>
       </c>
       <c r="CH2" t="n">
-        <v>226058</v>
+        <v>464251</v>
       </c>
       <c r="CI2" t="n">
-        <v>113282</v>
+        <v>110906</v>
       </c>
       <c r="CJ2" t="n">
-        <v>394212</v>
+        <v>531179</v>
       </c>
       <c r="CK2" t="n">
-        <v>162065</v>
+        <v>544727</v>
       </c>
       <c r="CL2" t="n">
-        <v>595300</v>
+        <v>428972</v>
       </c>
       <c r="CM2" t="n">
-        <v>104858</v>
+        <v>5689</v>
       </c>
       <c r="CN2" t="n">
-        <v>117416</v>
+        <v>770395</v>
       </c>
       <c r="CO2" t="n">
-        <v>697334</v>
+        <v>286885</v>
       </c>
       <c r="CP2" t="n">
-        <v>789881</v>
+        <v>116153</v>
       </c>
       <c r="CQ2" t="n">
-        <v>815861</v>
+        <v>183770</v>
       </c>
       <c r="CR2" t="n">
-        <v>200012</v>
+        <v>378175</v>
       </c>
       <c r="CS2" t="n">
-        <v>446426</v>
+        <v>746509</v>
       </c>
       <c r="CT2" t="n">
-        <v>66400</v>
+        <v>296740</v>
       </c>
       <c r="CU2" t="n">
-        <v>586946</v>
+        <v>571345</v>
       </c>
       <c r="CV2" t="n">
-        <v>467396</v>
+        <v>584266</v>
       </c>
     </row>
   </sheetData>
@@ -1544,7 +1544,7 @@
         <v>321</v>
       </c>
       <c r="B1" t="n">
-        <v>2294</v>
+        <v>856</v>
       </c>
     </row>
     <row r="2">
@@ -1583,42 +1583,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>9883</v>
+        <v>9885</v>
       </c>
       <c r="B1" t="n">
-        <v>25945</v>
+        <v>6729</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>834</v>
+        <v>46</v>
       </c>
       <c r="B2" t="n">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="C2" t="n">
-        <v>1097</v>
+        <v>1164</v>
       </c>
       <c r="D2" t="n">
-        <v>941</v>
+        <v>360</v>
       </c>
       <c r="E2" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>366</v>
+        <v>812</v>
       </c>
       <c r="G2" t="n">
-        <v>209</v>
+        <v>561</v>
       </c>
       <c r="H2" t="n">
-        <v>602</v>
+        <v>613</v>
       </c>
       <c r="I2" t="n">
-        <v>463</v>
+        <v>84</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>935</v>
       </c>
     </row>
   </sheetData>
@@ -1637,10 +1637,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>10203</v>
+        <v>10212</v>
       </c>
       <c r="B1" t="n">
-        <v>26085</v>
+        <v>6105</v>
       </c>
     </row>
     <row r="2">
@@ -1651,13 +1651,13 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>1247</v>
+        <v>1136</v>
       </c>
       <c r="D2" t="n">
-        <v>833</v>
+        <v>669</v>
       </c>
       <c r="E2" t="n">
-        <v>650</v>
+        <v>616</v>
       </c>
       <c r="F2" t="n">
         <v>179</v>
@@ -1669,10 +1669,10 @@
         <v>375</v>
       </c>
       <c r="I2" t="n">
-        <v>917</v>
+        <v>769</v>
       </c>
       <c r="J2" t="n">
-        <v>585</v>
+        <v>1051</v>
       </c>
     </row>
   </sheetData>
@@ -1691,72 +1691,72 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>17223</v>
+        <v>17253</v>
       </c>
       <c r="B1" t="n">
-        <v>117172</v>
+        <v>21959</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>7</v>
+        <v>405</v>
       </c>
       <c r="B2" t="n">
-        <v>152</v>
+        <v>1157</v>
       </c>
       <c r="C2" t="n">
-        <v>918</v>
+        <v>562</v>
       </c>
       <c r="D2" t="n">
-        <v>618</v>
+        <v>446</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>186</v>
+        <v>782</v>
       </c>
       <c r="G2" t="n">
-        <v>45</v>
+        <v>69</v>
       </c>
       <c r="H2" t="n">
-        <v>118</v>
+        <v>215</v>
       </c>
       <c r="I2" t="n">
-        <v>1347</v>
+        <v>763</v>
       </c>
       <c r="J2" t="n">
-        <v>791</v>
+        <v>1364</v>
       </c>
       <c r="K2" t="n">
-        <v>345</v>
+        <v>162</v>
       </c>
       <c r="L2" t="n">
-        <v>385</v>
+        <v>14</v>
       </c>
       <c r="M2" t="n">
-        <v>590</v>
+        <v>176</v>
       </c>
       <c r="N2" t="n">
-        <v>1332</v>
+        <v>1118</v>
       </c>
       <c r="O2" t="n">
-        <v>1132</v>
+        <v>730</v>
       </c>
       <c r="P2" t="n">
-        <v>789</v>
+        <v>1060</v>
       </c>
       <c r="Q2" t="n">
-        <v>510</v>
+        <v>483</v>
       </c>
       <c r="R2" t="n">
-        <v>1203</v>
+        <v>1363</v>
       </c>
       <c r="S2" t="n">
-        <v>1069</v>
+        <v>931</v>
       </c>
       <c r="T2" t="n">
-        <v>577</v>
+        <v>344</v>
       </c>
     </row>
   </sheetData>
@@ -1775,72 +1775,72 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>18031</v>
+        <v>17501</v>
       </c>
       <c r="B1" t="n">
-        <v>149632</v>
+        <v>25147</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>7</v>
+        <v>305</v>
       </c>
       <c r="B2" t="n">
-        <v>62</v>
+        <v>1260</v>
       </c>
       <c r="C2" t="n">
-        <v>449</v>
+        <v>755</v>
       </c>
       <c r="D2" t="n">
-        <v>596</v>
+        <v>413</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>104</v>
+        <v>19</v>
       </c>
       <c r="G2" t="n">
-        <v>299</v>
+        <v>554</v>
       </c>
       <c r="H2" t="n">
+        <v>173</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1371</v>
+      </c>
+      <c r="J2" t="n">
+        <v>608</v>
+      </c>
+      <c r="K2" t="n">
+        <v>864</v>
+      </c>
+      <c r="L2" t="n">
+        <v>204</v>
+      </c>
+      <c r="M2" t="n">
+        <v>385</v>
+      </c>
+      <c r="N2" t="n">
+        <v>1352</v>
+      </c>
+      <c r="O2" t="n">
+        <v>688</v>
+      </c>
+      <c r="P2" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>995</v>
+      </c>
+      <c r="R2" t="n">
+        <v>885</v>
+      </c>
+      <c r="S2" t="n">
+        <v>1129</v>
+      </c>
+      <c r="T2" t="n">
         <v>372</v>
-      </c>
-      <c r="I2" t="n">
-        <v>1385</v>
-      </c>
-      <c r="J2" t="n">
-        <v>911</v>
-      </c>
-      <c r="K2" t="n">
-        <v>786</v>
-      </c>
-      <c r="L2" t="n">
-        <v>439</v>
-      </c>
-      <c r="M2" t="n">
-        <v>584</v>
-      </c>
-      <c r="N2" t="n">
-        <v>1376</v>
-      </c>
-      <c r="O2" t="n">
-        <v>1191</v>
-      </c>
-      <c r="P2" t="n">
-        <v>909</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>829</v>
-      </c>
-      <c r="R2" t="n">
-        <v>1241</v>
-      </c>
-      <c r="S2" t="n">
-        <v>1107</v>
-      </c>
-      <c r="T2" t="n">
-        <v>275</v>
       </c>
     </row>
   </sheetData>
@@ -1859,10 +1859,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>94122</v>
+        <v>98363</v>
       </c>
       <c r="B1" t="n">
-        <v>63552</v>
+        <v>6773</v>
       </c>
     </row>
     <row r="2">
@@ -1876,13 +1876,13 @@
         <v>4829</v>
       </c>
       <c r="D2" t="n">
-        <v>7278</v>
+        <v>6855</v>
       </c>
       <c r="E2" t="n">
         <v>5204</v>
       </c>
       <c r="F2" t="n">
-        <v>8183</v>
+        <v>7981</v>
       </c>
       <c r="G2" t="n">
         <v>3140</v>
@@ -1891,7 +1891,7 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>8786</v>
+        <v>13652</v>
       </c>
       <c r="J2" t="n">
         <v>3829</v>
@@ -1913,42 +1913,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>94122</v>
+        <v>96328</v>
       </c>
       <c r="B1" t="n">
-        <v>53959</v>
+        <v>6094</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0</v>
+        <v>114</v>
       </c>
       <c r="B2" t="n">
-        <v>118</v>
+        <v>84</v>
       </c>
       <c r="C2" t="n">
-        <v>4829</v>
+        <v>4440</v>
       </c>
       <c r="D2" t="n">
-        <v>7278</v>
+        <v>6137</v>
       </c>
       <c r="E2" t="n">
-        <v>5204</v>
+        <v>4651</v>
       </c>
       <c r="F2" t="n">
-        <v>8183</v>
+        <v>8143</v>
       </c>
       <c r="G2" t="n">
-        <v>3140</v>
+        <v>11283</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>8786</v>
+        <v>2132</v>
       </c>
       <c r="J2" t="n">
-        <v>3829</v>
+        <v>6589</v>
       </c>
     </row>
   </sheetData>
@@ -1967,312 +1967,312 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>6318254</v>
+        <v>6309462</v>
       </c>
       <c r="B1" t="n">
-        <v>3651579</v>
+        <v>3609699</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>4719</v>
+        <v>112900</v>
       </c>
       <c r="B2" t="n">
-        <v>71268</v>
+        <v>89325</v>
       </c>
       <c r="C2" t="n">
-        <v>70778</v>
+        <v>1172</v>
       </c>
       <c r="D2" t="n">
-        <v>14873</v>
+        <v>74646</v>
       </c>
       <c r="E2" t="n">
-        <v>96495</v>
+        <v>41711</v>
       </c>
       <c r="F2" t="n">
-        <v>31497</v>
+        <v>3879</v>
       </c>
       <c r="G2" t="n">
-        <v>51628</v>
+        <v>22056</v>
       </c>
       <c r="H2" t="n">
-        <v>38548</v>
+        <v>38567</v>
       </c>
       <c r="I2" t="n">
-        <v>21114</v>
+        <v>70953</v>
       </c>
       <c r="J2" t="n">
-        <v>53817</v>
+        <v>25</v>
       </c>
       <c r="K2" t="n">
-        <v>55444</v>
+        <v>46591</v>
       </c>
       <c r="L2" t="n">
-        <v>105682</v>
+        <v>40629</v>
       </c>
       <c r="M2" t="n">
-        <v>123412</v>
+        <v>57609</v>
       </c>
       <c r="N2" t="n">
-        <v>7494</v>
+        <v>84928</v>
       </c>
       <c r="O2" t="n">
-        <v>100004</v>
+        <v>17047</v>
       </c>
       <c r="P2" t="n">
-        <v>72824</v>
+        <v>30024</v>
       </c>
       <c r="Q2" t="n">
-        <v>55638</v>
+        <v>92625</v>
       </c>
       <c r="R2" t="n">
-        <v>107666</v>
+        <v>65530</v>
       </c>
       <c r="S2" t="n">
-        <v>90980</v>
+        <v>69697</v>
       </c>
       <c r="T2" t="n">
-        <v>11666</v>
+        <v>22440</v>
       </c>
       <c r="U2" t="n">
-        <v>25346</v>
+        <v>80768</v>
       </c>
       <c r="V2" t="n">
-        <v>34601</v>
+        <v>104990</v>
       </c>
       <c r="W2" t="n">
+        <v>3274</v>
+      </c>
+      <c r="X2" t="n">
+        <v>30051</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>77340</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>104048</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>111458</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>36168</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>123050</v>
+      </c>
+      <c r="AD2" t="n">
         <v>0</v>
       </c>
-      <c r="X2" t="n">
-        <v>39945</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>37831</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>26444</v>
-      </c>
-      <c r="AA2" t="n">
-        <v>102260</v>
-      </c>
-      <c r="AB2" t="n">
-        <v>132224</v>
-      </c>
-      <c r="AC2" t="n">
-        <v>15443</v>
-      </c>
-      <c r="AD2" t="n">
-        <v>48606</v>
-      </c>
       <c r="AE2" t="n">
-        <v>43308</v>
+        <v>56</v>
       </c>
       <c r="AF2" t="n">
-        <v>2851</v>
+        <v>51915</v>
       </c>
       <c r="AG2" t="n">
-        <v>50996</v>
+        <v>58130</v>
       </c>
       <c r="AH2" t="n">
-        <v>97860</v>
+        <v>115234</v>
       </c>
       <c r="AI2" t="n">
-        <v>110473</v>
+        <v>8271</v>
       </c>
       <c r="AJ2" t="n">
-        <v>19256</v>
+        <v>29883</v>
       </c>
       <c r="AK2" t="n">
-        <v>6051</v>
+        <v>19782</v>
       </c>
       <c r="AL2" t="n">
-        <v>67030</v>
+        <v>79945</v>
       </c>
       <c r="AM2" t="n">
-        <v>87029</v>
+        <v>0</v>
       </c>
       <c r="AN2" t="n">
-        <v>56748</v>
+        <v>104770</v>
       </c>
       <c r="AO2" t="n">
-        <v>70321</v>
+        <v>49369</v>
       </c>
       <c r="AP2" t="n">
-        <v>120958</v>
+        <v>82864</v>
       </c>
       <c r="AQ2" t="n">
-        <v>83234</v>
+        <v>9574</v>
       </c>
       <c r="AR2" t="n">
-        <v>89916</v>
+        <v>119055</v>
       </c>
       <c r="AS2" t="n">
-        <v>14820</v>
+        <v>19345</v>
       </c>
       <c r="AT2" t="n">
-        <v>114996</v>
+        <v>121996</v>
       </c>
       <c r="AU2" t="n">
-        <v>100642</v>
+        <v>111307</v>
       </c>
       <c r="AV2" t="n">
-        <v>6326</v>
+        <v>77822</v>
       </c>
       <c r="AW2" t="n">
-        <v>132500</v>
+        <v>12939</v>
       </c>
       <c r="AX2" t="n">
-        <v>117206</v>
+        <v>96399</v>
       </c>
       <c r="AY2" t="n">
-        <v>61849</v>
+        <v>98883</v>
       </c>
       <c r="AZ2" t="n">
-        <v>26988</v>
+        <v>25157</v>
       </c>
       <c r="BA2" t="n">
-        <v>86316</v>
+        <v>115455</v>
       </c>
       <c r="BB2" t="n">
-        <v>12791</v>
+        <v>109916</v>
       </c>
       <c r="BC2" t="n">
-        <v>55484</v>
+        <v>6515</v>
       </c>
       <c r="BD2" t="n">
-        <v>0</v>
+        <v>59392</v>
       </c>
       <c r="BE2" t="n">
-        <v>20384</v>
+        <v>46486</v>
       </c>
       <c r="BF2" t="n">
-        <v>75893</v>
+        <v>63991</v>
       </c>
       <c r="BG2" t="n">
-        <v>62995</v>
+        <v>89010</v>
       </c>
       <c r="BH2" t="n">
-        <v>82833</v>
+        <v>42173</v>
       </c>
       <c r="BI2" t="n">
-        <v>95178</v>
+        <v>26003</v>
       </c>
       <c r="BJ2" t="n">
-        <v>80349</v>
+        <v>35255</v>
       </c>
       <c r="BK2" t="n">
-        <v>7833</v>
+        <v>119500</v>
       </c>
       <c r="BL2" t="n">
-        <v>85293</v>
+        <v>54994</v>
       </c>
       <c r="BM2" t="n">
-        <v>109009</v>
+        <v>84185</v>
       </c>
       <c r="BN2" t="n">
-        <v>31582</v>
+        <v>61417</v>
       </c>
       <c r="BO2" t="n">
-        <v>23786</v>
+        <v>12755</v>
       </c>
       <c r="BP2" t="n">
-        <v>21529</v>
+        <v>27016</v>
       </c>
       <c r="BQ2" t="n">
-        <v>43787</v>
+        <v>68894</v>
       </c>
       <c r="BR2" t="n">
-        <v>13646</v>
+        <v>18073</v>
       </c>
       <c r="BS2" t="n">
-        <v>28924</v>
+        <v>107209</v>
       </c>
       <c r="BT2" t="n">
-        <v>47370</v>
+        <v>24914</v>
       </c>
       <c r="BU2" t="n">
-        <v>59703</v>
+        <v>70394</v>
       </c>
       <c r="BV2" t="n">
-        <v>3343</v>
+        <v>16000</v>
       </c>
       <c r="BW2" t="n">
-        <v>45783</v>
+        <v>9193</v>
       </c>
       <c r="BX2" t="n">
-        <v>30113</v>
+        <v>6984</v>
       </c>
       <c r="BY2" t="n">
-        <v>120120</v>
+        <v>64678</v>
       </c>
       <c r="BZ2" t="n">
-        <v>104726</v>
+        <v>102102</v>
       </c>
       <c r="CA2" t="n">
-        <v>129735</v>
+        <v>73555</v>
       </c>
       <c r="CB2" t="n">
-        <v>7952</v>
+        <v>75682</v>
       </c>
       <c r="CC2" t="n">
-        <v>125476</v>
+        <v>88805</v>
       </c>
       <c r="CD2" t="n">
-        <v>17370</v>
+        <v>85455</v>
       </c>
       <c r="CE2" t="n">
-        <v>108434</v>
+        <v>29123</v>
       </c>
       <c r="CF2" t="n">
-        <v>74083</v>
+        <v>43965</v>
       </c>
       <c r="CG2" t="n">
-        <v>124195</v>
+        <v>96430</v>
       </c>
       <c r="CH2" t="n">
-        <v>37445</v>
+        <v>32555</v>
       </c>
       <c r="CI2" t="n">
-        <v>78746</v>
+        <v>54569</v>
       </c>
       <c r="CJ2" t="n">
-        <v>15417</v>
+        <v>35773</v>
       </c>
       <c r="CK2" t="n">
-        <v>66225</v>
+        <v>45454</v>
       </c>
       <c r="CL2" t="n">
-        <v>24</v>
+        <v>40905</v>
       </c>
       <c r="CM2" t="n">
-        <v>73832</v>
+        <v>93779</v>
       </c>
       <c r="CN2" t="n">
-        <v>78363</v>
+        <v>98838</v>
       </c>
       <c r="CO2" t="n">
-        <v>753</v>
+        <v>4206</v>
       </c>
       <c r="CP2" t="n">
-        <v>10982</v>
+        <v>67386</v>
       </c>
       <c r="CQ2" t="n">
-        <v>49300</v>
+        <v>124926</v>
       </c>
       <c r="CR2" t="n">
-        <v>31155</v>
+        <v>101390</v>
       </c>
       <c r="CS2" t="n">
-        <v>93283</v>
+        <v>92931</v>
       </c>
       <c r="CT2" t="n">
-        <v>35405</v>
+        <v>65240</v>
       </c>
       <c r="CU2" t="n">
-        <v>112838</v>
+        <v>14764</v>
       </c>
       <c r="CV2" t="n">
-        <v>64040</v>
+        <v>50204</v>
       </c>
     </row>
   </sheetData>

</xml_diff>